<commit_message>
atz planilha com dados da OCOR 2
</commit_message>
<xml_diff>
--- a/AZUVER_dashboard_data_2.xlsx
+++ b/AZUVER_dashboard_data_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srest\PycharmProjects\Dashboard_Informacional2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9123456-D840-475D-B245-839243D8B6C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10CB83E-5DA0-4C5E-8C4E-01DAFCB1138B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="relations_daily" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="325">
   <si>
     <t>data</t>
   </si>
@@ -1038,6 +1038,15 @@
   </si>
   <si>
     <t>Respostas às Aç de VERMELHO em busca de apoio ao MPL</t>
+  </si>
+  <si>
+    <t>Aliado</t>
+  </si>
+  <si>
+    <t>Dissuasão Dominante</t>
+  </si>
+  <si>
+    <t>Parceiro</t>
   </si>
 </sst>
 </file>
@@ -3859,7 +3868,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="30">
+    <row r="69" spans="1:9">
       <c r="A69" s="1">
         <v>45958</v>
       </c>
@@ -3870,15 +3879,15 @@
         <v>10</v>
       </c>
       <c r="D69">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="E69">
-        <v>62</v>
-      </c>
-      <c r="F69" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="G69" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="F69" t="s">
+        <v>80</v>
+      </c>
+      <c r="G69" t="s">
         <v>77</v>
       </c>
       <c r="H69" t="s">
@@ -3888,7 +3897,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="30">
+    <row r="70" spans="1:9">
       <c r="A70" s="1">
         <v>45958</v>
       </c>
@@ -3899,15 +3908,15 @@
         <v>10</v>
       </c>
       <c r="D70">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E70">
-        <v>65</v>
-      </c>
-      <c r="F70" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="F70" t="s">
         <v>11</v>
       </c>
-      <c r="G70" s="21" t="s">
+      <c r="G70" t="s">
         <v>77</v>
       </c>
       <c r="H70" t="s">
@@ -3917,7 +3926,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="30">
+    <row r="71" spans="1:9">
       <c r="A71" s="1">
         <v>45958</v>
       </c>
@@ -3928,16 +3937,16 @@
         <v>10</v>
       </c>
       <c r="D71">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E71">
-        <v>54</v>
-      </c>
-      <c r="F71" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G71" s="21" t="s">
-        <v>78</v>
+        <v>70</v>
+      </c>
+      <c r="F71" t="s">
+        <v>74</v>
+      </c>
+      <c r="G71" t="s">
+        <v>77</v>
       </c>
       <c r="H71" t="s">
         <v>12</v>
@@ -3946,7 +3955,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="30">
+    <row r="72" spans="1:9">
       <c r="A72" s="1">
         <v>45958</v>
       </c>
@@ -3962,10 +3971,10 @@
       <c r="E72">
         <v>51</v>
       </c>
-      <c r="F72" s="21" t="s">
+      <c r="F72" t="s">
         <v>11</v>
       </c>
-      <c r="G72" s="21" t="s">
+      <c r="G72" t="s">
         <v>78</v>
       </c>
       <c r="H72" t="s">
@@ -3975,7 +3984,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="30">
+    <row r="73" spans="1:9">
       <c r="A73" s="1">
         <v>45958</v>
       </c>
@@ -3991,10 +4000,10 @@
       <c r="E73">
         <v>61</v>
       </c>
-      <c r="F73" s="20" t="s">
+      <c r="F73" t="s">
         <v>75</v>
       </c>
-      <c r="G73" s="21" t="s">
+      <c r="G73" t="s">
         <v>77</v>
       </c>
       <c r="H73" t="s">
@@ -4004,7 +4013,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="30">
+    <row r="74" spans="1:9">
       <c r="A74" s="1">
         <v>45958</v>
       </c>
@@ -4015,16 +4024,16 @@
         <v>10</v>
       </c>
       <c r="D74">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="E74">
-        <v>64</v>
-      </c>
-      <c r="F74" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="G74" s="21" t="s">
-        <v>78</v>
+        <v>93</v>
+      </c>
+      <c r="F74" t="s">
+        <v>322</v>
+      </c>
+      <c r="G74" t="s">
+        <v>323</v>
       </c>
       <c r="H74" t="s">
         <v>12</v>
@@ -4033,7 +4042,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="30">
+    <row r="75" spans="1:9">
       <c r="A75" s="1">
         <v>45958</v>
       </c>
@@ -4049,10 +4058,10 @@
       <c r="E75">
         <v>58</v>
       </c>
-      <c r="F75" s="20" t="s">
+      <c r="F75" t="s">
         <v>74</v>
       </c>
-      <c r="G75" s="21" t="s">
+      <c r="G75" t="s">
         <v>78</v>
       </c>
       <c r="H75" t="s">
@@ -4062,7 +4071,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="30">
+    <row r="76" spans="1:9">
       <c r="A76" s="1">
         <v>45958</v>
       </c>
@@ -4073,15 +4082,15 @@
         <v>10</v>
       </c>
       <c r="D76">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="E76">
-        <v>50</v>
-      </c>
-      <c r="F76" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="G76" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="F76" t="s">
+        <v>80</v>
+      </c>
+      <c r="G76" t="s">
         <v>78</v>
       </c>
       <c r="H76" t="s">
@@ -4091,7 +4100,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="30">
+    <row r="77" spans="1:9">
       <c r="A77" s="1">
         <v>45958</v>
       </c>
@@ -4102,15 +4111,15 @@
         <v>10</v>
       </c>
       <c r="D77">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E77">
-        <v>61</v>
-      </c>
-      <c r="F77" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F77" t="s">
         <v>11</v>
       </c>
-      <c r="G77" s="21" t="s">
+      <c r="G77" t="s">
         <v>77</v>
       </c>
       <c r="H77" t="s">
@@ -4120,7 +4129,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="30">
+    <row r="78" spans="1:9">
       <c r="A78" s="1">
         <v>45958</v>
       </c>
@@ -4131,15 +4140,15 @@
         <v>10</v>
       </c>
       <c r="D78">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E78">
-        <v>61</v>
-      </c>
-      <c r="F78" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F78" t="s">
         <v>11</v>
       </c>
-      <c r="G78" s="21" t="s">
+      <c r="G78" t="s">
         <v>77</v>
       </c>
       <c r="H78" t="s">
@@ -4149,7 +4158,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="30">
+    <row r="79" spans="1:9">
       <c r="A79" s="1">
         <v>45958</v>
       </c>
@@ -4160,16 +4169,16 @@
         <v>10</v>
       </c>
       <c r="D79">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E79">
-        <v>52</v>
-      </c>
-      <c r="F79" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="G79" s="21" t="s">
-        <v>78</v>
+        <v>69</v>
+      </c>
+      <c r="F79" t="s">
+        <v>76</v>
+      </c>
+      <c r="G79" t="s">
+        <v>77</v>
       </c>
       <c r="H79" t="s">
         <v>12</v>
@@ -4178,7 +4187,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="30">
+    <row r="80" spans="1:9">
       <c r="A80" s="1">
         <v>45958</v>
       </c>
@@ -4189,15 +4198,15 @@
         <v>10</v>
       </c>
       <c r="D80">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E80">
-        <v>45</v>
-      </c>
-      <c r="F80" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="G80" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F80" t="s">
+        <v>75</v>
+      </c>
+      <c r="G80" t="s">
         <v>78</v>
       </c>
       <c r="H80" t="s">
@@ -4207,7 +4216,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="30">
+    <row r="81" spans="1:9">
       <c r="A81" s="1">
         <v>45958</v>
       </c>
@@ -4218,15 +4227,15 @@
         <v>10</v>
       </c>
       <c r="D81">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E81">
-        <v>47</v>
-      </c>
-      <c r="F81" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="G81" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="F81" t="s">
+        <v>11</v>
+      </c>
+      <c r="G81" t="s">
         <v>78</v>
       </c>
       <c r="H81" t="s">
@@ -4236,7 +4245,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="30">
+    <row r="82" spans="1:9">
       <c r="A82" s="1">
         <v>45958</v>
       </c>
@@ -4247,15 +4256,15 @@
         <v>10</v>
       </c>
       <c r="D82">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E82">
-        <v>66</v>
-      </c>
-      <c r="F82" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F82" t="s">
         <v>76</v>
       </c>
-      <c r="G82" s="21" t="s">
+      <c r="G82" t="s">
         <v>77</v>
       </c>
       <c r="H82" t="s">
@@ -4265,7 +4274,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="30">
+    <row r="83" spans="1:9">
       <c r="A83" s="1">
         <v>45958</v>
       </c>
@@ -4276,16 +4285,16 @@
         <v>10</v>
       </c>
       <c r="D83">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E83">
-        <v>72</v>
-      </c>
-      <c r="F83" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G83" s="21" t="s">
-        <v>77</v>
+        <v>86</v>
+      </c>
+      <c r="F83" t="s">
+        <v>76</v>
+      </c>
+      <c r="G83" t="s">
+        <v>323</v>
       </c>
       <c r="H83" t="s">
         <v>12</v>
@@ -4305,16 +4314,16 @@
         <v>10</v>
       </c>
       <c r="D84">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E84">
-        <v>34</v>
-      </c>
-      <c r="F84" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F84" t="s">
         <v>75</v>
       </c>
-      <c r="G84" s="21" t="s">
-        <v>79</v>
+      <c r="G84" t="s">
+        <v>78</v>
       </c>
       <c r="H84" t="s">
         <v>12</v>
@@ -4323,7 +4332,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="30">
+    <row r="85" spans="1:9">
       <c r="A85" s="1">
         <v>45958</v>
       </c>
@@ -4334,16 +4343,16 @@
         <v>14</v>
       </c>
       <c r="D85">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="E85">
-        <v>55</v>
-      </c>
-      <c r="F85" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="G85" s="21" t="s">
-        <v>78</v>
+        <v>74</v>
+      </c>
+      <c r="F85" t="s">
+        <v>324</v>
+      </c>
+      <c r="G85" t="s">
+        <v>77</v>
       </c>
       <c r="H85" t="s">
         <v>12</v>
@@ -4352,7 +4361,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="30">
+    <row r="86" spans="1:9">
       <c r="A86" s="1">
         <v>45958</v>
       </c>
@@ -4366,12 +4375,12 @@
         <v>60</v>
       </c>
       <c r="E86">
-        <v>62</v>
-      </c>
-      <c r="F86" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F86" t="s">
         <v>76</v>
       </c>
-      <c r="G86" s="21" t="s">
+      <c r="G86" t="s">
         <v>77</v>
       </c>
       <c r="H86" t="s">
@@ -4381,7 +4390,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="30">
+    <row r="87" spans="1:9">
       <c r="A87" s="1">
         <v>45958</v>
       </c>
@@ -4392,16 +4401,16 @@
         <v>14</v>
       </c>
       <c r="D87">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="E87">
-        <v>53</v>
-      </c>
-      <c r="F87" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G87" s="21" t="s">
-        <v>78</v>
+        <v>65</v>
+      </c>
+      <c r="F87" t="s">
+        <v>324</v>
+      </c>
+      <c r="G87" t="s">
+        <v>77</v>
       </c>
       <c r="H87" t="s">
         <v>12</v>
@@ -4410,7 +4419,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="30">
+    <row r="88" spans="1:9">
       <c r="A88" s="1">
         <v>45958</v>
       </c>
@@ -4421,15 +4430,15 @@
         <v>14</v>
       </c>
       <c r="D88">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E88">
-        <v>48</v>
-      </c>
-      <c r="F88" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F88" t="s">
         <v>75</v>
       </c>
-      <c r="G88" s="21" t="s">
+      <c r="G88" t="s">
         <v>78</v>
       </c>
       <c r="H88" t="s">
@@ -4439,7 +4448,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="30">
+    <row r="89" spans="1:9">
       <c r="A89" s="1">
         <v>45958</v>
       </c>
@@ -4450,15 +4459,15 @@
         <v>14</v>
       </c>
       <c r="D89">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E89">
-        <v>66</v>
-      </c>
-      <c r="F89" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="F89" t="s">
         <v>80</v>
       </c>
-      <c r="G89" s="21" t="s">
+      <c r="G89" t="s">
         <v>77</v>
       </c>
       <c r="H89" t="s">
@@ -4468,7 +4477,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="30">
+    <row r="90" spans="1:9">
       <c r="A90" s="1">
         <v>45958</v>
       </c>
@@ -4479,16 +4488,16 @@
         <v>14</v>
       </c>
       <c r="D90">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E90">
-        <v>43</v>
-      </c>
-      <c r="F90" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="G90" s="21" t="s">
-        <v>78</v>
+        <v>35</v>
+      </c>
+      <c r="F90" t="s">
+        <v>75</v>
+      </c>
+      <c r="G90" t="s">
+        <v>79</v>
       </c>
       <c r="H90" t="s">
         <v>12</v>
@@ -4497,7 +4506,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="30">
+    <row r="91" spans="1:9">
       <c r="A91" s="1">
         <v>45958</v>
       </c>
@@ -4513,10 +4522,10 @@
       <c r="E91">
         <v>59</v>
       </c>
-      <c r="F91" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="G91" s="21" t="s">
+      <c r="F91" t="s">
+        <v>80</v>
+      </c>
+      <c r="G91" t="s">
         <v>78</v>
       </c>
       <c r="H91" t="s">
@@ -4526,7 +4535,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="30">
+    <row r="92" spans="1:9">
       <c r="A92" s="1">
         <v>45958</v>
       </c>
@@ -4537,15 +4546,15 @@
         <v>14</v>
       </c>
       <c r="D92">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E92">
-        <v>50</v>
-      </c>
-      <c r="F92" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F92" t="s">
         <v>11</v>
       </c>
-      <c r="G92" s="21" t="s">
+      <c r="G92" t="s">
         <v>78</v>
       </c>
       <c r="H92" t="s">
@@ -4555,7 +4564,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="30">
+    <row r="93" spans="1:9">
       <c r="A93" s="1">
         <v>45958</v>
       </c>
@@ -4566,16 +4575,16 @@
         <v>14</v>
       </c>
       <c r="D93">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="E93">
-        <v>62</v>
-      </c>
-      <c r="F93" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G93" s="21" t="s">
-        <v>77</v>
+        <v>59</v>
+      </c>
+      <c r="F93" t="s">
+        <v>74</v>
+      </c>
+      <c r="G93" t="s">
+        <v>78</v>
       </c>
       <c r="H93" t="s">
         <v>12</v>
@@ -4584,7 +4593,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="30">
+    <row r="94" spans="1:9">
       <c r="A94" s="1">
         <v>45958</v>
       </c>
@@ -4595,16 +4604,16 @@
         <v>14</v>
       </c>
       <c r="D94">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E94">
-        <v>62</v>
-      </c>
-      <c r="F94" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G94" s="21" t="s">
-        <v>77</v>
+        <v>59</v>
+      </c>
+      <c r="F94" t="s">
+        <v>74</v>
+      </c>
+      <c r="G94" t="s">
+        <v>78</v>
       </c>
       <c r="H94" t="s">
         <v>12</v>
@@ -4613,7 +4622,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="30">
+    <row r="95" spans="1:9">
       <c r="A95" s="1">
         <v>45958</v>
       </c>
@@ -4624,15 +4633,15 @@
         <v>14</v>
       </c>
       <c r="D95">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="E95">
-        <v>51</v>
-      </c>
-      <c r="F95" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G95" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="F95" t="s">
+        <v>74</v>
+      </c>
+      <c r="G95" t="s">
         <v>78</v>
       </c>
       <c r="H95" t="s">
@@ -4642,7 +4651,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="30">
+    <row r="96" spans="1:9">
       <c r="A96" s="1">
         <v>45958</v>
       </c>
@@ -4653,16 +4662,16 @@
         <v>14</v>
       </c>
       <c r="D96">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="E96">
-        <v>52</v>
-      </c>
-      <c r="F96" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="G96" s="21" t="s">
-        <v>78</v>
+        <v>68</v>
+      </c>
+      <c r="F96" t="s">
+        <v>322</v>
+      </c>
+      <c r="G96" t="s">
+        <v>77</v>
       </c>
       <c r="H96" t="s">
         <v>12</v>
@@ -4671,7 +4680,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="30">
+    <row r="97" spans="1:9">
       <c r="A97" s="1">
         <v>45958</v>
       </c>
@@ -4682,15 +4691,15 @@
         <v>14</v>
       </c>
       <c r="D97">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E97">
         <v>50</v>
       </c>
-      <c r="F97" s="20" t="s">
+      <c r="F97" t="s">
         <v>74</v>
       </c>
-      <c r="G97" s="21" t="s">
+      <c r="G97" t="s">
         <v>78</v>
       </c>
       <c r="H97" t="s">
@@ -4700,7 +4709,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="30">
+    <row r="98" spans="1:9">
       <c r="A98" s="1">
         <v>45958</v>
       </c>
@@ -4711,15 +4720,15 @@
         <v>14</v>
       </c>
       <c r="D98">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E98">
-        <v>66</v>
-      </c>
-      <c r="F98" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G98" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F98" t="s">
+        <v>74</v>
+      </c>
+      <c r="G98" t="s">
         <v>77</v>
       </c>
       <c r="H98" t="s">
@@ -4729,7 +4738,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="30">
+    <row r="99" spans="1:9">
       <c r="A99" s="1">
         <v>45958</v>
       </c>
@@ -4740,16 +4749,16 @@
         <v>14</v>
       </c>
       <c r="D99">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="E99">
-        <v>73</v>
-      </c>
-      <c r="F99" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G99" s="21" t="s">
-        <v>77</v>
+        <v>85</v>
+      </c>
+      <c r="F99" t="s">
+        <v>322</v>
+      </c>
+      <c r="G99" t="s">
+        <v>323</v>
       </c>
       <c r="H99" t="s">
         <v>12</v>
@@ -4758,7 +4767,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="30">
+    <row r="100" spans="1:9">
       <c r="A100" s="1">
         <v>45958</v>
       </c>
@@ -4769,16 +4778,16 @@
         <v>14</v>
       </c>
       <c r="D100">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E100">
-        <v>56</v>
-      </c>
-      <c r="F100" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="G100" s="21" t="s">
-        <v>78</v>
+        <v>61</v>
+      </c>
+      <c r="F100" t="s">
+        <v>76</v>
+      </c>
+      <c r="G100" t="s">
+        <v>77</v>
       </c>
       <c r="H100" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
atz planilha com correção do cálculo e helper para calculo
</commit_message>
<xml_diff>
--- a/AZUVER_dashboard_data_2.xlsx
+++ b/AZUVER_dashboard_data_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srest\PycharmProjects\Dashboard_Informacional2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0BEB861-2543-4043-8CE0-49B71066976E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3B8402-5AAB-4030-9BD4-479EC79A1485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="333">
   <si>
     <t>data</t>
   </si>
@@ -1040,13 +1040,37 @@
     <t>Respostas às Aç de VERMELHO em busca de apoio ao MPL</t>
   </si>
   <si>
-    <t>Aliado</t>
-  </si>
-  <si>
-    <t>Dissuasão Dominante</t>
-  </si>
-  <si>
-    <t>Parceiro</t>
+    <t>Hostil (20–34)</t>
+  </si>
+  <si>
+    <t>Respeito/Temor Elevado (60–79)</t>
+  </si>
+  <si>
+    <t>Neutro (50–59)</t>
+  </si>
+  <si>
+    <t>Tenso/Desfavorável (35–49)</t>
+  </si>
+  <si>
+    <t>Respeito/Temor Moderado (40–59)</t>
+  </si>
+  <si>
+    <t>Hostilidade extrema (0–19)</t>
+  </si>
+  <si>
+    <t>Aliado (80–100)</t>
+  </si>
+  <si>
+    <t>Dissuasão Dominante (80–100)</t>
+  </si>
+  <si>
+    <t>Cooperativo (60–69)</t>
+  </si>
+  <si>
+    <t>Parceiro (70–79)</t>
+  </si>
+  <si>
+    <t>Respeito/Temor Baixo (20–39)</t>
   </si>
 </sst>
 </file>
@@ -1251,7 +1275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1304,11 +1328,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="24">
+    <dxf>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1607,7 +1637,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B7E38C3E-8A3D-4434-8337-0420E18C2416}" name="Tabela4" displayName="Tabela4" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B7E38C3E-8A3D-4434-8337-0420E18C2416}" name="Tabela4" displayName="Tabela4" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="23">
   <autoFilter ref="A1:I1048576" xr:uid="{B7E38C3E-8A3D-4434-8337-0420E18C2416}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{903F7B59-588A-4677-91D4-CAFFEF4BCC9C}" name="data"/>
@@ -1616,7 +1646,7 @@
     <tableColumn id="4" xr3:uid="{7F40A552-08DB-47E5-B8C9-D234A3618AC7}" name="R"/>
     <tableColumn id="5" xr3:uid="{6D524766-1B99-4A6B-BBB8-2C07618F12BD}" name="C"/>
     <tableColumn id="6" xr3:uid="{975C8660-93D0-4033-AA43-8AA370C045E9}" name="class_R"/>
-    <tableColumn id="7" xr3:uid="{B6DA6EC3-D88E-4812-89CE-2FD27455D195}" name="class_C"/>
+    <tableColumn id="7" xr3:uid="{B6DA6EC3-D88E-4812-89CE-2FD27455D195}" name="class_C" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{2DC65DDE-891F-45C1-A625-9C1EA845FBAC}" name="fonte_regra"/>
     <tableColumn id="9" xr3:uid="{ED276677-25B8-4FBE-A338-C1FDCB7FC603}" name="obs"/>
   </tableColumns>
@@ -1625,48 +1655,48 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A3AD564-B18D-4439-A198-8AF944A99772}" name="tblActors" displayName="tblActors" ref="A1:D17" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19" totalsRowBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A3AD564-B18D-4439-A198-8AF944A99772}" name="tblActors" displayName="tblActors" ref="A1:D17" totalsRowShown="0" headerRowDxfId="22" headerRowBorderDxfId="21" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A1:D17" xr:uid="{5A3AD564-B18D-4439-A198-8AF944A99772}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3122FF93-D7C9-47C4-AAE7-E5CBE0FA3A54}" name="actor_id" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{2220D84D-1A4B-4A12-888A-7592053EDECC}" name="nome" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{7244E1B6-C06A-46BA-A29E-7198716E593E}" name="tipo" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{10B1B0CA-D667-4698-9FAC-A50EC4C9BE0A}" name="cluster_opcional" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{3122FF93-D7C9-47C4-AAE7-E5CBE0FA3A54}" name="actor_id" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{2220D84D-1A4B-4A12-888A-7592053EDECC}" name="nome" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{7244E1B6-C06A-46BA-A29E-7198716E593E}" name="tipo" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{10B1B0CA-D667-4698-9FAC-A50EC4C9BE0A}" name="cluster_opcional" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8EE140BC-D0AD-4653-A557-FEB72E7706BB}" name="Tabela3" displayName="Tabela3" ref="A1:H279" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8EE140BC-D0AD-4653-A557-FEB72E7706BB}" name="Tabela3" displayName="Tabela3" ref="A1:H279" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A1:H279" xr:uid="{8EE140BC-D0AD-4653-A557-FEB72E7706BB}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{A64D0630-7FB4-4675-AF15-DFA9CC4C3218}" name="event_id"/>
     <tableColumn id="2" xr3:uid="{ABB220E9-794F-4B06-80FB-EA100148E885}" name="data"/>
-    <tableColumn id="3" xr3:uid="{DEFA5E68-941A-4720-891C-051748ACEEE4}" name="titulo" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{2AA18C9F-BAB7-429C-BD76-624D918E02A6}" name="descricao" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{ACAD5301-D426-46EE-A7F5-46CA1210DCDF}" name="tipo" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{C20CACB4-38DD-423C-80F3-2EAB1574530A}" name="tags" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{46484C08-2E71-4200-A22E-BF604C745824}" name="fonte" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{9B6E38A2-36A7-42AA-A46E-F35C16B84F1E}" name="responsabilidade" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{DEFA5E68-941A-4720-891C-051748ACEEE4}" name="titulo" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{2AA18C9F-BAB7-429C-BD76-624D918E02A6}" name="descricao" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{ACAD5301-D426-46EE-A7F5-46CA1210DCDF}" name="tipo" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{C20CACB4-38DD-423C-80F3-2EAB1574530A}" name="tags" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{46484C08-2E71-4200-A22E-BF604C745824}" name="fonte" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{9B6E38A2-36A7-42AA-A46E-F35C16B84F1E}" name="responsabilidade" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8F935928-F61E-454D-9EE9-3D2DFF7048F4}" name="Tabela2" displayName="Tabela2" ref="A1:K327" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="3" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8F935928-F61E-454D-9EE9-3D2DFF7048F4}" name="Tabela2" displayName="Tabela2" ref="A1:K327" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
   <autoFilter ref="A1:K327" xr:uid="{8F935928-F61E-454D-9EE9-3D2DFF7048F4}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{BAF761B8-D6AF-48D3-A1F5-3D35088A4234}" name="event_id"/>
-    <tableColumn id="2" xr3:uid="{78C225EA-4EED-44B0-BBCE-FD76B432B72B}" name="actor_id" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{78C225EA-4EED-44B0-BBCE-FD76B432B72B}" name="actor_id" dataDxfId="2">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(C2, tblActors[nome], tblActors[actor_id], ""), "")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{37AE2979-DF01-47CD-BEA5-BA034C5B3757}" name="actor_name"/>
     <tableColumn id="4" xr3:uid="{7BDACF9C-965E-4CCF-94CF-242CB57A4AC1}" name="partido"/>
     <tableColumn id="5" xr3:uid="{6A802EC2-6140-4C9F-9D92-0F2B0C6B0D2F}" name="delta_R"/>
     <tableColumn id="6" xr3:uid="{5830257E-D8FA-438E-9298-17ED813D6C77}" name="delta_C"/>
-    <tableColumn id="7" xr3:uid="{ED6BE6E1-B0BE-4C05-8C17-6A8218AD71A0}" name="racional" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{ED6BE6E1-B0BE-4C05-8C17-6A8218AD71A0}" name="racional" dataDxfId="1"/>
     <tableColumn id="8" xr3:uid="{481A5440-CA6F-4A3B-984A-1D2FFA263532}" name="atraso_dias"/>
     <tableColumn id="9" xr3:uid="{DD506A33-5271-4DFF-AAA8-7F12E055CCD0}" name="delta_opiniao_direta"/>
     <tableColumn id="10" xr3:uid="{9B94DE7A-D5B7-427A-A880-C7C51E771C9F}" name="delta_midia"/>
@@ -1961,14 +1991,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.5703125" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.7109375" style="14" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2901,7 +2931,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="30">
+    <row r="33" spans="1:11" ht="30">
       <c r="A33" s="1">
         <v>45946</v>
       </c>
@@ -2930,17 +2960,17 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:11">
       <c r="A34" s="1"/>
       <c r="F34" s="20"/>
       <c r="G34" s="21"/>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:11">
       <c r="A35" s="1"/>
       <c r="F35" s="20"/>
       <c r="G35" s="21"/>
     </row>
-    <row r="36" spans="1:9" ht="30">
+    <row r="36" spans="1:11" ht="30">
       <c r="A36" s="1">
         <v>45952</v>
       </c>
@@ -2969,7 +2999,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="30">
+    <row r="37" spans="1:11" ht="30">
       <c r="A37" s="1">
         <v>45952</v>
       </c>
@@ -2998,7 +3028,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="30">
+    <row r="38" spans="1:11" ht="30">
       <c r="A38" s="1">
         <v>45952</v>
       </c>
@@ -3026,8 +3056,12 @@
       <c r="I38" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" ht="30">
+      <c r="K38">
+        <f>Tabela4[[#This Row],[R]]-25</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="30">
       <c r="A39" s="1">
         <v>45952</v>
       </c>
@@ -3056,7 +3090,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="30">
+    <row r="40" spans="1:11" ht="30">
       <c r="A40" s="1">
         <v>45952</v>
       </c>
@@ -3085,7 +3119,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="30">
+    <row r="41" spans="1:11" ht="30">
       <c r="A41" s="1">
         <v>45952</v>
       </c>
@@ -3114,7 +3148,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="30">
+    <row r="42" spans="1:11" ht="30">
       <c r="A42" s="1">
         <v>45952</v>
       </c>
@@ -3143,7 +3177,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="30">
+    <row r="43" spans="1:11" ht="30">
       <c r="A43" s="1">
         <v>45952</v>
       </c>
@@ -3172,7 +3206,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="30">
+    <row r="44" spans="1:11" ht="30">
       <c r="A44" s="1">
         <v>45952</v>
       </c>
@@ -3201,7 +3235,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="30">
+    <row r="45" spans="1:11" ht="30">
       <c r="A45" s="1">
         <v>45952</v>
       </c>
@@ -3230,7 +3264,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="30">
+    <row r="46" spans="1:11" ht="30">
       <c r="A46" s="1">
         <v>45952</v>
       </c>
@@ -3259,7 +3293,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="30">
+    <row r="47" spans="1:11" ht="30">
       <c r="A47" s="1">
         <v>45952</v>
       </c>
@@ -3288,7 +3322,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="30">
+    <row r="48" spans="1:11" ht="30">
       <c r="A48" s="1">
         <v>45952</v>
       </c>
@@ -3868,7 +3902,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
+    <row r="69" spans="1:9" ht="30">
       <c r="A69" s="1">
         <v>45958</v>
       </c>
@@ -3879,16 +3913,16 @@
         <v>10</v>
       </c>
       <c r="D69">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E69">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F69" t="s">
-        <v>80</v>
-      </c>
-      <c r="G69" t="s">
-        <v>77</v>
+        <v>322</v>
+      </c>
+      <c r="G69" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H69" t="s">
         <v>12</v>
@@ -3897,7 +3931,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="70" spans="1:9">
+    <row r="70" spans="1:9" ht="30">
       <c r="A70" s="1">
         <v>45958</v>
       </c>
@@ -3908,16 +3942,16 @@
         <v>10</v>
       </c>
       <c r="D70">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E70">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F70" t="s">
-        <v>11</v>
-      </c>
-      <c r="G70" t="s">
-        <v>77</v>
+        <v>324</v>
+      </c>
+      <c r="G70" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H70" t="s">
         <v>12</v>
@@ -3926,7 +3960,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
+    <row r="71" spans="1:9" ht="30">
       <c r="A71" s="1">
         <v>45958</v>
       </c>
@@ -3937,16 +3971,16 @@
         <v>10</v>
       </c>
       <c r="D71">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E71">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F71" t="s">
-        <v>74</v>
-      </c>
-      <c r="G71" t="s">
-        <v>77</v>
+        <v>325</v>
+      </c>
+      <c r="G71" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H71" t="s">
         <v>12</v>
@@ -3955,7 +3989,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
+    <row r="72" spans="1:9" ht="30">
       <c r="A72" s="1">
         <v>45958</v>
       </c>
@@ -3972,10 +4006,10 @@
         <v>51</v>
       </c>
       <c r="F72" t="s">
-        <v>11</v>
-      </c>
-      <c r="G72" t="s">
-        <v>78</v>
+        <v>324</v>
+      </c>
+      <c r="G72" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H72" t="s">
         <v>12</v>
@@ -3984,7 +4018,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
+    <row r="73" spans="1:9" ht="30">
       <c r="A73" s="1">
         <v>45958</v>
       </c>
@@ -3995,16 +4029,16 @@
         <v>10</v>
       </c>
       <c r="D73">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E73">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F73" t="s">
-        <v>75</v>
-      </c>
-      <c r="G73" t="s">
-        <v>77</v>
+        <v>327</v>
+      </c>
+      <c r="G73" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H73" t="s">
         <v>12</v>
@@ -4013,7 +4047,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="74" spans="1:9">
+    <row r="74" spans="1:9" ht="30">
       <c r="A74" s="1">
         <v>45958</v>
       </c>
@@ -4024,16 +4058,16 @@
         <v>10</v>
       </c>
       <c r="D74">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E74">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F74" t="s">
-        <v>322</v>
-      </c>
-      <c r="G74" t="s">
-        <v>323</v>
+        <v>328</v>
+      </c>
+      <c r="G74" s="14" t="s">
+        <v>329</v>
       </c>
       <c r="H74" t="s">
         <v>12</v>
@@ -4042,7 +4076,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="75" spans="1:9">
+    <row r="75" spans="1:9" ht="30">
       <c r="A75" s="1">
         <v>45958</v>
       </c>
@@ -4059,10 +4093,10 @@
         <v>58</v>
       </c>
       <c r="F75" t="s">
-        <v>74</v>
-      </c>
-      <c r="G75" t="s">
-        <v>78</v>
+        <v>325</v>
+      </c>
+      <c r="G75" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H75" t="s">
         <v>12</v>
@@ -4071,7 +4105,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="76" spans="1:9">
+    <row r="76" spans="1:9" ht="30">
       <c r="A76" s="1">
         <v>45958</v>
       </c>
@@ -4088,10 +4122,10 @@
         <v>54</v>
       </c>
       <c r="F76" t="s">
-        <v>80</v>
-      </c>
-      <c r="G76" t="s">
-        <v>78</v>
+        <v>322</v>
+      </c>
+      <c r="G76" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H76" t="s">
         <v>12</v>
@@ -4100,7 +4134,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="77" spans="1:9">
+    <row r="77" spans="1:9" ht="30">
       <c r="A77" s="1">
         <v>45958</v>
       </c>
@@ -4111,16 +4145,16 @@
         <v>10</v>
       </c>
       <c r="D77">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E77">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F77" t="s">
-        <v>11</v>
-      </c>
-      <c r="G77" t="s">
-        <v>77</v>
+        <v>324</v>
+      </c>
+      <c r="G77" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H77" t="s">
         <v>12</v>
@@ -4129,7 +4163,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="78" spans="1:9">
+    <row r="78" spans="1:9" ht="30">
       <c r="A78" s="1">
         <v>45958</v>
       </c>
@@ -4140,16 +4174,16 @@
         <v>10</v>
       </c>
       <c r="D78">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E78">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F78" t="s">
-        <v>11</v>
-      </c>
-      <c r="G78" t="s">
-        <v>77</v>
+        <v>324</v>
+      </c>
+      <c r="G78" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H78" t="s">
         <v>12</v>
@@ -4158,7 +4192,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="79" spans="1:9">
+    <row r="79" spans="1:9" ht="30">
       <c r="A79" s="1">
         <v>45958</v>
       </c>
@@ -4175,10 +4209,10 @@
         <v>69</v>
       </c>
       <c r="F79" t="s">
-        <v>76</v>
-      </c>
-      <c r="G79" t="s">
-        <v>77</v>
+        <v>330</v>
+      </c>
+      <c r="G79" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H79" t="s">
         <v>12</v>
@@ -4187,7 +4221,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="80" spans="1:9">
+    <row r="80" spans="1:9" ht="30">
       <c r="A80" s="1">
         <v>45958</v>
       </c>
@@ -4204,10 +4238,10 @@
         <v>59</v>
       </c>
       <c r="F80" t="s">
-        <v>75</v>
-      </c>
-      <c r="G80" t="s">
-        <v>78</v>
+        <v>327</v>
+      </c>
+      <c r="G80" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H80" t="s">
         <v>12</v>
@@ -4216,7 +4250,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="81" spans="1:9">
+    <row r="81" spans="1:9" ht="30">
       <c r="A81" s="1">
         <v>45958</v>
       </c>
@@ -4233,10 +4267,10 @@
         <v>51</v>
       </c>
       <c r="F81" t="s">
-        <v>11</v>
-      </c>
-      <c r="G81" t="s">
-        <v>78</v>
+        <v>324</v>
+      </c>
+      <c r="G81" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H81" t="s">
         <v>12</v>
@@ -4245,7 +4279,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="82" spans="1:9">
+    <row r="82" spans="1:9" ht="30">
       <c r="A82" s="1">
         <v>45958</v>
       </c>
@@ -4256,16 +4290,16 @@
         <v>10</v>
       </c>
       <c r="D82">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E82">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F82" t="s">
-        <v>76</v>
-      </c>
-      <c r="G82" t="s">
-        <v>77</v>
+        <v>330</v>
+      </c>
+      <c r="G82" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H82" t="s">
         <v>12</v>
@@ -4274,7 +4308,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="83" spans="1:9">
+    <row r="83" spans="1:9" ht="30">
       <c r="A83" s="1">
         <v>45958</v>
       </c>
@@ -4285,16 +4319,16 @@
         <v>10</v>
       </c>
       <c r="D83">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E83">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F83" t="s">
-        <v>76</v>
-      </c>
-      <c r="G83" t="s">
-        <v>323</v>
+        <v>331</v>
+      </c>
+      <c r="G83" s="14" t="s">
+        <v>329</v>
       </c>
       <c r="H83" t="s">
         <v>12</v>
@@ -4303,7 +4337,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="84" spans="1:9">
+    <row r="84" spans="1:9" ht="30">
       <c r="A84" s="1">
         <v>45958</v>
       </c>
@@ -4320,10 +4354,10 @@
         <v>48</v>
       </c>
       <c r="F84" t="s">
-        <v>75</v>
-      </c>
-      <c r="G84" t="s">
-        <v>78</v>
+        <v>327</v>
+      </c>
+      <c r="G84" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H84" t="s">
         <v>12</v>
@@ -4332,7 +4366,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="85" spans="1:9">
+    <row r="85" spans="1:9" ht="30">
       <c r="A85" s="1">
         <v>45958</v>
       </c>
@@ -4349,10 +4383,10 @@
         <v>74</v>
       </c>
       <c r="F85" t="s">
-        <v>324</v>
-      </c>
-      <c r="G85" t="s">
-        <v>77</v>
+        <v>331</v>
+      </c>
+      <c r="G85" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H85" t="s">
         <v>12</v>
@@ -4361,7 +4395,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="86" spans="1:9">
+    <row r="86" spans="1:9" ht="30">
       <c r="A86" s="1">
         <v>45958</v>
       </c>
@@ -4378,10 +4412,10 @@
         <v>68</v>
       </c>
       <c r="F86" t="s">
-        <v>76</v>
-      </c>
-      <c r="G86" t="s">
-        <v>77</v>
+        <v>330</v>
+      </c>
+      <c r="G86" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H86" t="s">
         <v>12</v>
@@ -4390,7 +4424,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="87" spans="1:9">
+    <row r="87" spans="1:9" ht="30">
       <c r="A87" s="1">
         <v>45958</v>
       </c>
@@ -4407,10 +4441,10 @@
         <v>65</v>
       </c>
       <c r="F87" t="s">
-        <v>324</v>
-      </c>
-      <c r="G87" t="s">
-        <v>77</v>
+        <v>331</v>
+      </c>
+      <c r="G87" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H87" t="s">
         <v>12</v>
@@ -4419,7 +4453,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="88" spans="1:9">
+    <row r="88" spans="1:9" ht="30">
       <c r="A88" s="1">
         <v>45958</v>
       </c>
@@ -4436,10 +4470,10 @@
         <v>50</v>
       </c>
       <c r="F88" t="s">
-        <v>75</v>
-      </c>
-      <c r="G88" t="s">
-        <v>78</v>
+        <v>327</v>
+      </c>
+      <c r="G88" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H88" t="s">
         <v>12</v>
@@ -4448,7 +4482,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="89" spans="1:9">
+    <row r="89" spans="1:9" ht="30">
       <c r="A89" s="1">
         <v>45958</v>
       </c>
@@ -4465,10 +4499,10 @@
         <v>69</v>
       </c>
       <c r="F89" t="s">
-        <v>80</v>
-      </c>
-      <c r="G89" t="s">
-        <v>77</v>
+        <v>322</v>
+      </c>
+      <c r="G89" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H89" t="s">
         <v>12</v>
@@ -4477,7 +4511,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="90" spans="1:9">
+    <row r="90" spans="1:9" ht="30">
       <c r="A90" s="1">
         <v>45958</v>
       </c>
@@ -4494,10 +4528,10 @@
         <v>35</v>
       </c>
       <c r="F90" t="s">
-        <v>75</v>
-      </c>
-      <c r="G90" t="s">
-        <v>79</v>
+        <v>327</v>
+      </c>
+      <c r="G90" s="14" t="s">
+        <v>332</v>
       </c>
       <c r="H90" t="s">
         <v>12</v>
@@ -4506,7 +4540,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="91" spans="1:9">
+    <row r="91" spans="1:9" ht="30">
       <c r="A91" s="1">
         <v>45958</v>
       </c>
@@ -4523,10 +4557,10 @@
         <v>59</v>
       </c>
       <c r="F91" t="s">
-        <v>80</v>
-      </c>
-      <c r="G91" t="s">
-        <v>78</v>
+        <v>322</v>
+      </c>
+      <c r="G91" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H91" t="s">
         <v>12</v>
@@ -4535,7 +4569,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="92" spans="1:9">
+    <row r="92" spans="1:9" ht="30">
       <c r="A92" s="1">
         <v>45958</v>
       </c>
@@ -4552,10 +4586,10 @@
         <v>48</v>
       </c>
       <c r="F92" t="s">
-        <v>11</v>
-      </c>
-      <c r="G92" t="s">
-        <v>78</v>
+        <v>324</v>
+      </c>
+      <c r="G92" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H92" t="s">
         <v>12</v>
@@ -4564,7 +4598,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="93" spans="1:9">
+    <row r="93" spans="1:9" ht="30">
       <c r="A93" s="1">
         <v>45958</v>
       </c>
@@ -4581,10 +4615,10 @@
         <v>59</v>
       </c>
       <c r="F93" t="s">
-        <v>74</v>
-      </c>
-      <c r="G93" t="s">
-        <v>78</v>
+        <v>325</v>
+      </c>
+      <c r="G93" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H93" t="s">
         <v>12</v>
@@ -4593,7 +4627,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="94" spans="1:9">
+    <row r="94" spans="1:9" ht="30">
       <c r="A94" s="1">
         <v>45958</v>
       </c>
@@ -4610,10 +4644,10 @@
         <v>59</v>
       </c>
       <c r="F94" t="s">
-        <v>74</v>
-      </c>
-      <c r="G94" t="s">
-        <v>78</v>
+        <v>325</v>
+      </c>
+      <c r="G94" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H94" t="s">
         <v>12</v>
@@ -4622,7 +4656,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="95" spans="1:9">
+    <row r="95" spans="1:9" ht="30">
       <c r="A95" s="1">
         <v>45958</v>
       </c>
@@ -4639,10 +4673,10 @@
         <v>53</v>
       </c>
       <c r="F95" t="s">
-        <v>74</v>
-      </c>
-      <c r="G95" t="s">
-        <v>78</v>
+        <v>325</v>
+      </c>
+      <c r="G95" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H95" t="s">
         <v>12</v>
@@ -4651,7 +4685,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="96" spans="1:9">
+    <row r="96" spans="1:9" ht="30">
       <c r="A96" s="1">
         <v>45958</v>
       </c>
@@ -4668,10 +4702,10 @@
         <v>68</v>
       </c>
       <c r="F96" t="s">
-        <v>322</v>
-      </c>
-      <c r="G96" t="s">
-        <v>77</v>
+        <v>328</v>
+      </c>
+      <c r="G96" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H96" t="s">
         <v>12</v>
@@ -4680,7 +4714,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
+    <row r="97" spans="1:9" ht="30">
       <c r="A97" s="1">
         <v>45958</v>
       </c>
@@ -4697,10 +4731,10 @@
         <v>50</v>
       </c>
       <c r="F97" t="s">
-        <v>74</v>
-      </c>
-      <c r="G97" t="s">
-        <v>78</v>
+        <v>325</v>
+      </c>
+      <c r="G97" s="14" t="s">
+        <v>326</v>
       </c>
       <c r="H97" t="s">
         <v>12</v>
@@ -4709,7 +4743,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:9" ht="30">
       <c r="A98" s="1">
         <v>45958</v>
       </c>
@@ -4726,10 +4760,10 @@
         <v>68</v>
       </c>
       <c r="F98" t="s">
-        <v>74</v>
-      </c>
-      <c r="G98" t="s">
-        <v>77</v>
+        <v>325</v>
+      </c>
+      <c r="G98" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H98" t="s">
         <v>12</v>
@@ -4738,7 +4772,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="99" spans="1:9">
+    <row r="99" spans="1:9" ht="30">
       <c r="A99" s="1">
         <v>45958</v>
       </c>
@@ -4749,16 +4783,16 @@
         <v>14</v>
       </c>
       <c r="D99">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E99">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F99" t="s">
-        <v>322</v>
-      </c>
-      <c r="G99" t="s">
-        <v>323</v>
+        <v>328</v>
+      </c>
+      <c r="G99" s="14" t="s">
+        <v>329</v>
       </c>
       <c r="H99" t="s">
         <v>12</v>
@@ -4767,7 +4801,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="100" spans="1:9">
+    <row r="100" spans="1:9" ht="30">
       <c r="A100" s="1">
         <v>45958</v>
       </c>
@@ -4784,10 +4818,10 @@
         <v>61</v>
       </c>
       <c r="F100" t="s">
-        <v>76</v>
-      </c>
-      <c r="G100" t="s">
-        <v>77</v>
+        <v>330</v>
+      </c>
+      <c r="G100" s="14" t="s">
+        <v>323</v>
       </c>
       <c r="H100" t="s">
         <v>12</v>
@@ -5152,7 +5186,7 @@
         <v>33</v>
       </c>
       <c r="B3" s="1">
-        <v>45952.486111111109</v>
+        <v>45952</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>259</v>
@@ -6319,10 +6353,10 @@
       <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="24">
         <v>-2</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="24">
         <v>0</v>
       </c>
       <c r="G2" s="14" t="s">
@@ -6346,10 +6380,10 @@
       <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
+      <c r="E3" s="24">
+        <v>0</v>
+      </c>
+      <c r="F3" s="24">
         <v>0</v>
       </c>
       <c r="G3" s="14" t="s">
@@ -6373,10 +6407,10 @@
       <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="24">
         <v>-4</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="24">
         <v>1</v>
       </c>
       <c r="G4" s="14" t="s">
@@ -6400,10 +6434,10 @@
       <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="24">
         <v>-2</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="24">
         <v>0</v>
       </c>
       <c r="G5" s="14" t="s">
@@ -6427,10 +6461,10 @@
       <c r="D6" t="s">
         <v>14</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="24">
         <v>3</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="24">
         <v>2</v>
       </c>
       <c r="G6" s="14" t="s">
@@ -6454,10 +6488,10 @@
       <c r="D7" t="s">
         <v>14</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="24">
         <v>-8</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="24">
         <v>-7</v>
       </c>
       <c r="G7" s="14" t="s">
@@ -6481,10 +6515,10 @@
       <c r="D8" t="s">
         <v>14</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="24">
         <v>-4</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="24">
         <v>3</v>
       </c>
       <c r="G8" s="14" t="s">
@@ -6508,10 +6542,10 @@
       <c r="D9" t="s">
         <v>14</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
+      <c r="E9" s="24">
+        <v>0</v>
+      </c>
+      <c r="F9" s="24">
         <v>0</v>
       </c>
       <c r="G9" s="14" t="s">
@@ -6535,10 +6569,10 @@
       <c r="D10" t="s">
         <v>14</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="24">
         <v>-3</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="24">
         <v>2</v>
       </c>
       <c r="G10" s="14" t="s">
@@ -6562,10 +6596,10 @@
       <c r="D11" t="s">
         <v>14</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="24">
         <v>-3</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="24">
         <v>2</v>
       </c>
       <c r="G11" s="14" t="s">
@@ -6589,10 +6623,10 @@
       <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
+      <c r="E12" s="24">
+        <v>0</v>
+      </c>
+      <c r="F12" s="24">
         <v>3</v>
       </c>
       <c r="G12" s="14" t="s">
@@ -6616,10 +6650,10 @@
       <c r="D13" t="s">
         <v>14</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="24">
         <v>8</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="24">
         <v>7</v>
       </c>
       <c r="G13" s="14" t="s">
@@ -6643,10 +6677,10 @@
       <c r="D14" t="s">
         <v>14</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="24">
         <v>3</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="24">
         <v>2</v>
       </c>
       <c r="G14" s="14" t="s">
@@ -6670,10 +6704,10 @@
       <c r="D15" t="s">
         <v>14</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="24">
         <v>-2</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="24">
         <v>3</v>
       </c>
       <c r="G15" s="14" t="s">
@@ -6697,10 +6731,10 @@
       <c r="D16" t="s">
         <v>14</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="24">
         <v>3</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="24">
         <v>3</v>
       </c>
       <c r="G16" s="14" t="s">
@@ -6724,10 +6758,10 @@
       <c r="D17" t="s">
         <v>14</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="24">
         <v>7</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="24">
         <v>6</v>
       </c>
       <c r="G17" s="14" t="s">
@@ -6751,10 +6785,10 @@
       <c r="D18" t="s">
         <v>10</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="24">
         <v>1</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="24">
         <v>2</v>
       </c>
       <c r="G18" s="14" t="s">
@@ -6778,10 +6812,10 @@
       <c r="D19" t="s">
         <v>10</v>
       </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-      <c r="F19">
+      <c r="E19" s="24">
+        <v>0</v>
+      </c>
+      <c r="F19" s="24">
         <v>0</v>
       </c>
       <c r="G19" s="14" t="s">
@@ -6805,10 +6839,10 @@
       <c r="D20" t="s">
         <v>10</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="24">
         <v>5</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="24">
         <v>4</v>
       </c>
       <c r="G20" s="14" t="s">
@@ -6832,10 +6866,10 @@
       <c r="D21" t="s">
         <v>10</v>
       </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21">
+      <c r="E21" s="24">
+        <v>0</v>
+      </c>
+      <c r="F21" s="24">
         <v>1</v>
       </c>
       <c r="G21" s="14" t="s">
@@ -6859,10 +6893,10 @@
       <c r="D22" t="s">
         <v>10</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="24">
         <v>-3</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="24">
         <v>1</v>
       </c>
       <c r="G22" s="14" t="s">
@@ -6886,10 +6920,10 @@
       <c r="D23" t="s">
         <v>10</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="24">
         <v>9</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="24">
         <v>9</v>
       </c>
       <c r="G23" s="18" t="s">
@@ -6913,10 +6947,10 @@
       <c r="D24" t="s">
         <v>10</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="24">
         <v>3</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="24">
         <v>0</v>
       </c>
       <c r="G24" s="14" t="s">
@@ -6940,10 +6974,10 @@
       <c r="D25" t="s">
         <v>10</v>
       </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
+      <c r="E25" s="24">
+        <v>0</v>
+      </c>
+      <c r="F25" s="24">
         <v>0</v>
       </c>
       <c r="G25" s="14" t="s">
@@ -6967,10 +7001,10 @@
       <c r="D26" t="s">
         <v>10</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="24">
         <v>1</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="24">
         <v>1</v>
       </c>
       <c r="G26" s="14" t="s">
@@ -6994,10 +7028,10 @@
       <c r="D27" t="s">
         <v>10</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="24">
         <v>1</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="24">
         <v>1</v>
       </c>
       <c r="G27" s="14" t="s">
@@ -7021,10 +7055,10 @@
       <c r="D28" t="s">
         <v>10</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="24">
         <v>3</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="24">
         <v>2</v>
       </c>
       <c r="G28" s="14" t="s">
@@ -7048,10 +7082,10 @@
       <c r="D29" t="s">
         <v>10</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="24">
         <v>-4</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="24">
         <v>0</v>
       </c>
       <c r="G29" s="14" t="s">
@@ -7075,10 +7109,10 @@
       <c r="D30" t="s">
         <v>10</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="24">
         <v>3</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="24">
         <v>2</v>
       </c>
       <c r="G30" s="14" t="s">
@@ -7102,10 +7136,10 @@
       <c r="D31" t="s">
         <v>10</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="24">
         <v>1</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="24">
         <v>1</v>
       </c>
       <c r="G31" s="18" t="s">
@@ -7129,10 +7163,10 @@
       <c r="D32" t="s">
         <v>10</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="24">
         <v>5</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="24">
         <v>4</v>
       </c>
       <c r="G32" s="14" t="s">
@@ -7156,10 +7190,10 @@
       <c r="D33" t="s">
         <v>10</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="24">
         <v>-2</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="24">
         <v>1</v>
       </c>
       <c r="G33" s="14" t="s">
@@ -7183,14 +7217,17 @@
       <c r="D34" t="s">
         <v>10</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="24">
         <v>4</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="24">
         <v>3</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="30">
@@ -7207,14 +7244,17 @@
       <c r="D35" t="s">
         <v>10</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="24">
         <v>3</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="24">
         <v>2</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="30">
@@ -7231,14 +7271,17 @@
       <c r="D36" t="s">
         <v>10</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="24">
         <v>-6</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="24">
         <v>5</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="30">
@@ -7255,14 +7298,17 @@
       <c r="D37" t="s">
         <v>10</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="24">
         <v>3</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="24">
         <v>3</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30">
@@ -7279,14 +7325,17 @@
       <c r="D38" t="s">
         <v>10</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="24">
         <v>3</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="24">
         <v>3</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="30">
@@ -7303,14 +7352,17 @@
       <c r="D39" t="s">
         <v>10</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="24">
         <v>3</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="24">
         <v>3</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="30">
@@ -7327,14 +7379,17 @@
       <c r="D40" t="s">
         <v>10</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="24">
         <v>3</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="24">
         <v>3</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="30">
@@ -7351,14 +7406,17 @@
       <c r="D41" t="s">
         <v>10</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="24">
         <v>1</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="24">
         <v>2</v>
       </c>
       <c r="G41" s="14" t="s">
         <v>292</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="30">
@@ -7375,14 +7433,17 @@
       <c r="D42" t="s">
         <v>10</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="24">
         <v>-7</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="24">
         <v>3</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>299</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="30">
@@ -7399,14 +7460,17 @@
       <c r="D43" t="s">
         <v>14</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="24">
         <v>8</v>
       </c>
-      <c r="F43">
+      <c r="F43" s="24">
         <v>4</v>
       </c>
       <c r="G43" s="14" t="s">
         <v>299</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="30">
@@ -7423,14 +7487,17 @@
       <c r="D44" t="s">
         <v>10</v>
       </c>
-      <c r="E44" s="23">
+      <c r="E44" s="24">
         <v>6</v>
       </c>
-      <c r="F44" s="23">
+      <c r="F44" s="24">
         <v>5</v>
       </c>
       <c r="G44" s="14" t="s">
         <v>299</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="30">
@@ -7447,14 +7514,17 @@
       <c r="D45" t="s">
         <v>14</v>
       </c>
-      <c r="E45" s="23">
+      <c r="E45" s="24">
         <v>2</v>
       </c>
-      <c r="F45" s="23">
+      <c r="F45" s="24">
         <v>1</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>299</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="30">
@@ -7471,14 +7541,17 @@
       <c r="D46" t="s">
         <v>10</v>
       </c>
-      <c r="E46" s="23">
+      <c r="E46" s="24">
         <v>3</v>
       </c>
-      <c r="F46" s="23">
+      <c r="F46" s="24">
         <v>4</v>
       </c>
       <c r="G46" s="14" t="s">
         <v>299</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30">
@@ -7495,14 +7568,17 @@
       <c r="D47" t="s">
         <v>14</v>
       </c>
-      <c r="E47" s="23">
+      <c r="E47" s="24">
         <v>4</v>
       </c>
-      <c r="F47" s="23">
+      <c r="F47" s="24">
         <v>2</v>
       </c>
       <c r="G47" s="14" t="s">
         <v>299</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="30">
@@ -7519,17 +7595,20 @@
       <c r="D48" t="s">
         <v>10</v>
       </c>
-      <c r="E48" s="23">
+      <c r="E48" s="24">
         <v>5</v>
       </c>
-      <c r="F48" s="23">
+      <c r="F48" s="24">
         <v>5</v>
       </c>
       <c r="G48" s="14" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" ht="30">
+      <c r="H48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="30">
       <c r="A49" t="s">
         <v>82</v>
       </c>
@@ -7543,17 +7622,20 @@
       <c r="D49" t="s">
         <v>14</v>
       </c>
-      <c r="E49" s="23">
+      <c r="E49" s="24">
         <v>-7</v>
       </c>
-      <c r="F49" s="23">
+      <c r="F49" s="24">
         <v>-2</v>
       </c>
       <c r="G49" s="14" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" ht="30">
+      <c r="H49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="30">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -7567,17 +7649,20 @@
       <c r="D50" t="s">
         <v>10</v>
       </c>
-      <c r="E50" s="23">
+      <c r="E50" s="24">
         <v>5</v>
       </c>
-      <c r="F50" s="23">
+      <c r="F50" s="24">
         <v>4</v>
       </c>
       <c r="G50" s="14" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" ht="30">
+      <c r="H50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="30">
       <c r="A51" t="s">
         <v>82</v>
       </c>
@@ -7591,17 +7676,20 @@
       <c r="D51" t="s">
         <v>14</v>
       </c>
-      <c r="E51" s="23">
+      <c r="E51" s="24">
         <v>-4</v>
       </c>
-      <c r="F51" s="23">
+      <c r="F51" s="24">
         <v>0</v>
       </c>
       <c r="G51" s="14" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" ht="30">
+      <c r="H51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="30">
       <c r="A52" t="s">
         <v>82</v>
       </c>
@@ -7615,17 +7703,20 @@
       <c r="D52" t="s">
         <v>10</v>
       </c>
-      <c r="E52" s="23">
+      <c r="E52" s="24">
         <v>-6</v>
       </c>
-      <c r="F52" s="23">
+      <c r="F52" s="24">
         <v>6</v>
       </c>
       <c r="G52" s="14" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" ht="30">
+      <c r="H52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="30">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -7639,17 +7730,20 @@
       <c r="D53" t="s">
         <v>14</v>
       </c>
-      <c r="E53" s="23">
+      <c r="E53" s="24">
         <v>2</v>
       </c>
-      <c r="F53" s="23">
+      <c r="F53" s="24">
         <v>0</v>
       </c>
       <c r="G53" s="14" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" ht="30">
+      <c r="H53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="30">
       <c r="A54" t="s">
         <v>83</v>
       </c>
@@ -7663,17 +7757,20 @@
       <c r="D54" t="s">
         <v>10</v>
       </c>
-      <c r="E54" s="23">
+      <c r="E54" s="24">
         <v>3</v>
       </c>
-      <c r="F54" s="23">
+      <c r="F54" s="24">
         <v>3</v>
       </c>
       <c r="G54" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" ht="30">
+      <c r="H54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="30">
       <c r="A55" t="s">
         <v>83</v>
       </c>
@@ -7687,17 +7784,20 @@
       <c r="D55" t="s">
         <v>10</v>
       </c>
-      <c r="E55" s="23">
+      <c r="E55" s="24">
         <v>5</v>
       </c>
-      <c r="F55" s="23">
+      <c r="F55" s="24">
         <v>3</v>
       </c>
       <c r="G55" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" ht="30">
+      <c r="H55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="30">
       <c r="A56" t="s">
         <v>83</v>
       </c>
@@ -7711,17 +7811,20 @@
       <c r="D56" t="s">
         <v>10</v>
       </c>
-      <c r="E56" s="23">
+      <c r="E56" s="24">
         <v>3</v>
       </c>
-      <c r="F56" s="23">
+      <c r="F56" s="24">
         <v>2</v>
       </c>
       <c r="G56" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" ht="30">
+      <c r="H56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="30">
       <c r="A57" t="s">
         <v>83</v>
       </c>
@@ -7735,17 +7838,20 @@
       <c r="D57" t="s">
         <v>10</v>
       </c>
-      <c r="E57" s="23">
+      <c r="E57" s="24">
         <v>3</v>
       </c>
-      <c r="F57" s="23">
+      <c r="F57" s="24">
         <v>2</v>
       </c>
       <c r="G57" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" ht="30">
+      <c r="H57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="30">
       <c r="A58" t="s">
         <v>83</v>
       </c>
@@ -7759,17 +7865,20 @@
       <c r="D58" t="s">
         <v>10</v>
       </c>
-      <c r="E58" s="23">
+      <c r="E58" s="24">
         <v>5</v>
       </c>
-      <c r="F58" s="23">
+      <c r="F58" s="24">
         <v>3</v>
       </c>
       <c r="G58" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" ht="30">
+      <c r="H58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="30">
       <c r="A59" t="s">
         <v>83</v>
       </c>
@@ -7783,17 +7892,20 @@
       <c r="D59" t="s">
         <v>10</v>
       </c>
-      <c r="E59" s="23">
+      <c r="E59" s="24">
         <v>-6</v>
       </c>
-      <c r="F59" s="23">
+      <c r="F59" s="24">
         <v>0</v>
       </c>
       <c r="G59" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" ht="30">
+      <c r="H59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="30">
       <c r="A60" t="s">
         <v>83</v>
       </c>
@@ -7807,17 +7919,20 @@
       <c r="D60" t="s">
         <v>10</v>
       </c>
-      <c r="E60" s="23">
+      <c r="E60" s="24">
         <v>4</v>
       </c>
-      <c r="F60" s="23">
+      <c r="F60" s="24">
         <v>4</v>
       </c>
       <c r="G60" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" ht="30">
+      <c r="H60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="30">
       <c r="A61" t="s">
         <v>83</v>
       </c>
@@ -7831,17 +7946,20 @@
       <c r="D61" t="s">
         <v>10</v>
       </c>
-      <c r="E61" s="23">
-        <v>0</v>
-      </c>
-      <c r="F61" s="23">
+      <c r="E61" s="24">
+        <v>0</v>
+      </c>
+      <c r="F61" s="24">
         <v>0</v>
       </c>
       <c r="G61" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" ht="30">
+      <c r="H61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="30">
       <c r="A62" t="s">
         <v>83</v>
       </c>
@@ -7855,17 +7973,20 @@
       <c r="D62" t="s">
         <v>14</v>
       </c>
-      <c r="E62" s="23">
+      <c r="E62" s="24">
         <v>4</v>
       </c>
-      <c r="F62" s="23">
+      <c r="F62" s="24">
         <v>1</v>
       </c>
       <c r="G62" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" ht="30">
+      <c r="H62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="30">
       <c r="A63" t="s">
         <v>83</v>
       </c>
@@ -7879,17 +8000,20 @@
       <c r="D63" t="s">
         <v>14</v>
       </c>
-      <c r="E63" s="23">
+      <c r="E63" s="24">
         <v>6</v>
       </c>
-      <c r="F63" s="23">
+      <c r="F63" s="24">
         <v>2</v>
       </c>
       <c r="G63" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" ht="30">
+      <c r="H63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="30">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -7903,17 +8027,20 @@
       <c r="D64" t="s">
         <v>14</v>
       </c>
-      <c r="E64" s="23">
+      <c r="E64" s="24">
         <v>-2</v>
       </c>
-      <c r="F64" s="23">
+      <c r="F64" s="24">
         <v>-2</v>
       </c>
       <c r="G64" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" ht="30">
+      <c r="H64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="30">
       <c r="A65" t="s">
         <v>83</v>
       </c>
@@ -7927,17 +8054,20 @@
       <c r="D65" t="s">
         <v>14</v>
       </c>
-      <c r="E65" s="23">
+      <c r="E65" s="24">
         <v>-2</v>
       </c>
-      <c r="F65" s="23">
+      <c r="F65" s="24">
         <v>-2</v>
       </c>
       <c r="G65" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" ht="30">
+      <c r="H65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="30">
       <c r="A66" t="s">
         <v>83</v>
       </c>
@@ -7951,17 +8081,20 @@
       <c r="D66" t="s">
         <v>14</v>
       </c>
-      <c r="E66" s="23">
+      <c r="E66" s="24">
         <v>-6</v>
       </c>
-      <c r="F66" s="23">
+      <c r="F66" s="24">
         <v>-2</v>
       </c>
       <c r="G66" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" ht="30">
+      <c r="H66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="30">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -7975,17 +8108,20 @@
       <c r="D67" t="s">
         <v>14</v>
       </c>
-      <c r="E67" s="23">
+      <c r="E67" s="24">
         <v>8</v>
       </c>
-      <c r="F67" s="23">
+      <c r="F67" s="24">
         <v>3</v>
       </c>
       <c r="G67" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" ht="30">
+      <c r="H67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="30">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -7999,17 +8135,20 @@
       <c r="D68" t="s">
         <v>14</v>
       </c>
-      <c r="E68" s="23">
+      <c r="E68" s="24">
         <v>-5</v>
       </c>
-      <c r="F68" s="23">
+      <c r="F68" s="24">
         <v>-2</v>
       </c>
       <c r="G68" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" ht="30">
+      <c r="H68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="30">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -8023,17 +8162,20 @@
       <c r="D69" t="s">
         <v>14</v>
       </c>
-      <c r="E69" s="23">
+      <c r="E69" s="24">
         <v>2</v>
       </c>
-      <c r="F69" s="23">
+      <c r="F69" s="24">
         <v>2</v>
       </c>
       <c r="G69" s="14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" ht="30">
+      <c r="H69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="30">
       <c r="A70" t="s">
         <v>84</v>
       </c>
@@ -8047,17 +8189,20 @@
       <c r="D70" t="s">
         <v>10</v>
       </c>
-      <c r="E70" s="23">
+      <c r="E70" s="24">
         <v>-10</v>
       </c>
-      <c r="F70" s="23">
+      <c r="F70" s="24">
         <v>6</v>
       </c>
       <c r="G70" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" ht="30">
+      <c r="H70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="30">
       <c r="A71" t="s">
         <v>84</v>
       </c>
@@ -8071,17 +8216,20 @@
       <c r="D71" t="s">
         <v>10</v>
       </c>
-      <c r="E71" s="23">
+      <c r="E71" s="24">
         <v>-2</v>
       </c>
-      <c r="F71" s="23">
+      <c r="F71" s="24">
         <v>4</v>
       </c>
       <c r="G71" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" ht="30">
+      <c r="H71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="30">
       <c r="A72" t="s">
         <v>84</v>
       </c>
@@ -8095,17 +8243,20 @@
       <c r="D72" t="s">
         <v>10</v>
       </c>
-      <c r="E72" s="23">
+      <c r="E72" s="24">
         <v>-2</v>
       </c>
-      <c r="F72" s="23">
+      <c r="F72" s="24">
         <v>4</v>
       </c>
       <c r="G72" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" ht="30">
+      <c r="H72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" ht="30">
       <c r="A73" t="s">
         <v>84</v>
       </c>
@@ -8119,17 +8270,20 @@
       <c r="D73" t="s">
         <v>10</v>
       </c>
-      <c r="E73" s="23">
+      <c r="E73" s="24">
         <v>-2</v>
       </c>
-      <c r="F73" s="23">
+      <c r="F73" s="24">
         <v>4</v>
       </c>
       <c r="G73" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" ht="30">
+      <c r="H73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="30">
       <c r="A74" t="s">
         <v>84</v>
       </c>
@@ -8143,17 +8297,20 @@
       <c r="D74" t="s">
         <v>10</v>
       </c>
-      <c r="E74" s="23">
+      <c r="E74" s="24">
         <v>-2</v>
       </c>
-      <c r="F74" s="23">
+      <c r="F74" s="24">
         <v>4</v>
       </c>
       <c r="G74" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" ht="30">
+      <c r="H74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="30">
       <c r="A75" t="s">
         <v>84</v>
       </c>
@@ -8167,17 +8324,20 @@
       <c r="D75" t="s">
         <v>10</v>
       </c>
-      <c r="E75" s="23">
+      <c r="E75" s="24">
         <v>8</v>
       </c>
-      <c r="F75" s="23">
+      <c r="F75" s="24">
         <v>7</v>
       </c>
       <c r="G75" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" ht="30">
+      <c r="H75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="30">
       <c r="A76" t="s">
         <v>84</v>
       </c>
@@ -8191,17 +8351,20 @@
       <c r="D76" t="s">
         <v>10</v>
       </c>
-      <c r="E76" s="23">
+      <c r="E76" s="24">
         <v>7</v>
       </c>
-      <c r="F76" s="23">
+      <c r="F76" s="24">
         <v>8</v>
       </c>
       <c r="G76" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" ht="30">
+      <c r="H76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="30">
       <c r="A77" t="s">
         <v>84</v>
       </c>
@@ -8215,17 +8378,20 @@
       <c r="D77" t="s">
         <v>10</v>
       </c>
-      <c r="E77" s="23">
+      <c r="E77" s="24">
         <v>-8</v>
       </c>
-      <c r="F77" s="23">
+      <c r="F77" s="24">
         <v>5</v>
       </c>
       <c r="G77" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="78" spans="1:7" ht="30">
+      <c r="H77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="30">
       <c r="A78" t="s">
         <v>84</v>
       </c>
@@ -8239,17 +8405,20 @@
       <c r="D78" t="s">
         <v>10</v>
       </c>
-      <c r="E78" s="23">
+      <c r="E78" s="24">
         <v>-10</v>
       </c>
-      <c r="F78" s="23">
+      <c r="F78" s="24">
         <v>2</v>
       </c>
       <c r="G78" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" ht="30">
+      <c r="H78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="30">
       <c r="A79" t="s">
         <v>84</v>
       </c>
@@ -8263,17 +8432,20 @@
       <c r="D79" t="s">
         <v>14</v>
       </c>
-      <c r="E79" s="23">
+      <c r="E79" s="24">
         <v>8</v>
       </c>
-      <c r="F79" s="23">
+      <c r="F79" s="24">
         <v>4</v>
       </c>
       <c r="G79" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" ht="30">
+      <c r="H79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" ht="30">
       <c r="A80" t="s">
         <v>84</v>
       </c>
@@ -8287,17 +8459,20 @@
       <c r="D80" t="s">
         <v>14</v>
       </c>
-      <c r="E80" s="23">
+      <c r="E80" s="24">
         <v>-2</v>
       </c>
-      <c r="F80" s="23">
+      <c r="F80" s="24">
         <v>4</v>
       </c>
       <c r="G80" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" ht="30">
+      <c r="H80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" ht="30">
       <c r="A81" t="s">
         <v>84</v>
       </c>
@@ -8311,17 +8486,20 @@
       <c r="D81" t="s">
         <v>14</v>
       </c>
-      <c r="E81" s="23">
+      <c r="E81" s="24">
         <v>-2</v>
       </c>
-      <c r="F81" s="23">
+      <c r="F81" s="24">
         <v>4</v>
       </c>
       <c r="G81" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" ht="30">
+      <c r="H81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="30">
       <c r="A82" t="s">
         <v>84</v>
       </c>
@@ -8335,17 +8513,20 @@
       <c r="D82" t="s">
         <v>14</v>
       </c>
-      <c r="E82" s="23">
+      <c r="E82" s="24">
         <v>-2</v>
       </c>
-      <c r="F82" s="23">
+      <c r="F82" s="24">
         <v>4</v>
       </c>
       <c r="G82" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" ht="30">
+      <c r="H82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="30">
       <c r="A83" t="s">
         <v>84</v>
       </c>
@@ -8359,17 +8540,20 @@
       <c r="D83" t="s">
         <v>14</v>
       </c>
-      <c r="E83" s="23">
+      <c r="E83" s="24">
         <v>-2</v>
       </c>
-      <c r="F83" s="23">
+      <c r="F83" s="24">
         <v>4</v>
       </c>
       <c r="G83" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" ht="30">
+      <c r="H83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="30">
       <c r="A84" t="s">
         <v>84</v>
       </c>
@@ -8383,17 +8567,20 @@
       <c r="D84" t="s">
         <v>14</v>
       </c>
-      <c r="E84" s="23">
+      <c r="E84" s="24">
         <v>-9</v>
       </c>
-      <c r="F84" s="23">
+      <c r="F84" s="24">
         <v>4</v>
       </c>
       <c r="G84" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" ht="30">
+      <c r="H84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" ht="30">
       <c r="A85" t="s">
         <v>84</v>
       </c>
@@ -8407,17 +8594,20 @@
       <c r="D85" t="s">
         <v>14</v>
       </c>
-      <c r="E85" s="23">
+      <c r="E85" s="24">
         <v>-10</v>
       </c>
-      <c r="F85" s="23">
+      <c r="F85" s="24">
         <v>2</v>
       </c>
       <c r="G85" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" ht="30">
+      <c r="H85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="30">
       <c r="A86" t="s">
         <v>84</v>
       </c>
@@ -8431,17 +8621,20 @@
       <c r="D86" t="s">
         <v>14</v>
       </c>
-      <c r="E86" s="23">
+      <c r="E86" s="24">
         <v>-8</v>
       </c>
-      <c r="F86" s="23">
+      <c r="F86" s="24">
         <v>5</v>
       </c>
       <c r="G86" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" ht="30">
+      <c r="H86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" ht="30">
       <c r="A87" t="s">
         <v>84</v>
       </c>
@@ -8455,17 +8648,20 @@
       <c r="D87" t="s">
         <v>14</v>
       </c>
-      <c r="E87" s="23">
+      <c r="E87" s="24">
         <v>7</v>
       </c>
-      <c r="F87" s="23">
+      <c r="F87" s="24">
         <v>8</v>
       </c>
       <c r="G87" s="14" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" ht="30">
+      <c r="H87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" ht="30">
       <c r="A88" t="s">
         <v>85</v>
       </c>
@@ -8479,17 +8675,20 @@
       <c r="D88" t="s">
         <v>10</v>
       </c>
-      <c r="E88" s="23">
+      <c r="E88" s="24">
         <v>6</v>
       </c>
-      <c r="F88" s="23">
+      <c r="F88" s="24">
         <v>9</v>
       </c>
       <c r="G88" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" ht="30">
+      <c r="H88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" ht="30">
       <c r="A89" t="s">
         <v>85</v>
       </c>
@@ -8503,17 +8702,20 @@
       <c r="D89" t="s">
         <v>10</v>
       </c>
-      <c r="E89" s="23">
+      <c r="E89" s="24">
         <v>-10</v>
       </c>
-      <c r="F89" s="23">
+      <c r="F89" s="24">
         <v>8</v>
       </c>
       <c r="G89" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" ht="30">
+      <c r="H89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" ht="30">
       <c r="A90" t="s">
         <v>85</v>
       </c>
@@ -8527,17 +8729,20 @@
       <c r="D90" t="s">
         <v>10</v>
       </c>
-      <c r="E90" s="23">
+      <c r="E90" s="24">
         <v>-8</v>
       </c>
-      <c r="F90" s="23">
+      <c r="F90" s="24">
         <v>8</v>
       </c>
       <c r="G90" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" ht="30">
+      <c r="H90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" ht="30">
       <c r="A91" t="s">
         <v>85</v>
       </c>
@@ -8551,17 +8756,20 @@
       <c r="D91" t="s">
         <v>10</v>
       </c>
-      <c r="E91" s="23">
+      <c r="E91" s="24">
         <v>-4</v>
       </c>
-      <c r="F91" s="23">
+      <c r="F91" s="24">
         <v>5</v>
       </c>
       <c r="G91" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" ht="30">
+      <c r="H91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" ht="30">
       <c r="A92" t="s">
         <v>85</v>
       </c>
@@ -8575,17 +8783,20 @@
       <c r="D92" t="s">
         <v>10</v>
       </c>
-      <c r="E92" s="23">
+      <c r="E92" s="24">
         <v>-7</v>
       </c>
-      <c r="F92" s="23">
+      <c r="F92" s="24">
         <v>8</v>
       </c>
       <c r="G92" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="93" spans="1:7" ht="30">
+      <c r="H92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" ht="30">
       <c r="A93" t="s">
         <v>85</v>
       </c>
@@ -8599,17 +8810,20 @@
       <c r="D93" t="s">
         <v>14</v>
       </c>
-      <c r="E93" s="23">
-        <v>0</v>
-      </c>
-      <c r="F93" s="23">
+      <c r="E93" s="24">
+        <v>0</v>
+      </c>
+      <c r="F93" s="24">
         <v>0</v>
       </c>
       <c r="G93" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" ht="30">
+      <c r="H93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" ht="30">
       <c r="A94" t="s">
         <v>85</v>
       </c>
@@ -8623,17 +8837,20 @@
       <c r="D94" t="s">
         <v>14</v>
       </c>
-      <c r="E94" s="23">
+      <c r="E94" s="24">
         <v>-5</v>
       </c>
-      <c r="F94" s="23">
+      <c r="F94" s="24">
         <v>6</v>
       </c>
       <c r="G94" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="95" spans="1:7" ht="30">
+      <c r="H94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" ht="30">
       <c r="A95" t="s">
         <v>85</v>
       </c>
@@ -8647,17 +8864,20 @@
       <c r="D95" t="s">
         <v>14</v>
       </c>
-      <c r="E95" s="23">
-        <v>0</v>
-      </c>
-      <c r="F95" s="23">
+      <c r="E95" s="24">
+        <v>0</v>
+      </c>
+      <c r="F95" s="24">
         <v>-4</v>
       </c>
       <c r="G95" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="96" spans="1:7" ht="30">
+      <c r="H95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" ht="30">
       <c r="A96" t="s">
         <v>85</v>
       </c>
@@ -8671,17 +8891,20 @@
       <c r="D96" t="s">
         <v>14</v>
       </c>
-      <c r="E96" s="23">
+      <c r="E96" s="24">
         <v>-2</v>
       </c>
-      <c r="F96" s="23">
+      <c r="F96" s="24">
         <v>-4</v>
       </c>
       <c r="G96" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="97" spans="1:7" ht="30">
+      <c r="H96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" ht="30">
       <c r="A97" t="s">
         <v>85</v>
       </c>
@@ -8695,17 +8918,20 @@
       <c r="D97" t="s">
         <v>14</v>
       </c>
-      <c r="E97" s="23">
-        <v>0</v>
-      </c>
-      <c r="F97" s="23">
+      <c r="E97" s="24">
+        <v>0</v>
+      </c>
+      <c r="F97" s="24">
         <v>-3</v>
       </c>
       <c r="G97" s="14" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="98" spans="1:7" ht="30">
+      <c r="H97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" ht="30">
       <c r="A98" t="s">
         <v>90</v>
       </c>
@@ -8719,17 +8945,20 @@
       <c r="D98" t="s">
         <v>10</v>
       </c>
-      <c r="E98" s="23">
+      <c r="E98" s="24">
         <v>-7</v>
       </c>
-      <c r="F98" s="23">
+      <c r="F98" s="24">
         <v>2</v>
       </c>
       <c r="G98" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="99" spans="1:7" ht="30">
+      <c r="H98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" ht="30">
       <c r="A99" t="s">
         <v>90</v>
       </c>
@@ -8743,17 +8972,20 @@
       <c r="D99" t="s">
         <v>10</v>
       </c>
-      <c r="E99" s="23">
+      <c r="E99" s="24">
         <v>-6</v>
       </c>
-      <c r="F99" s="23">
+      <c r="F99" s="24">
         <v>2</v>
       </c>
       <c r="G99" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="100" spans="1:7" ht="30">
+      <c r="H99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="30">
       <c r="A100" t="s">
         <v>90</v>
       </c>
@@ -8767,17 +8999,20 @@
       <c r="D100" t="s">
         <v>10</v>
       </c>
-      <c r="E100" s="23">
+      <c r="E100" s="24">
         <v>2</v>
       </c>
-      <c r="F100" s="23">
+      <c r="F100" s="24">
         <v>1</v>
       </c>
       <c r="G100" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="101" spans="1:7" ht="30">
+      <c r="H100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="30">
       <c r="A101" t="s">
         <v>90</v>
       </c>
@@ -8791,17 +9026,20 @@
       <c r="D101" t="s">
         <v>10</v>
       </c>
-      <c r="E101" s="23">
+      <c r="E101" s="24">
         <v>2</v>
       </c>
-      <c r="F101" s="23">
+      <c r="F101" s="24">
         <v>1</v>
       </c>
       <c r="G101" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="102" spans="1:7" ht="30">
+      <c r="H101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="30">
       <c r="A102" t="s">
         <v>90</v>
       </c>
@@ -8815,17 +9053,20 @@
       <c r="D102" t="s">
         <v>10</v>
       </c>
-      <c r="E102" s="23">
+      <c r="E102" s="24">
         <v>5</v>
       </c>
-      <c r="F102" s="23">
+      <c r="F102" s="24">
         <v>4</v>
       </c>
       <c r="G102" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="103" spans="1:7" ht="30">
+      <c r="H102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" ht="30">
       <c r="A103" t="s">
         <v>90</v>
       </c>
@@ -8839,17 +9080,20 @@
       <c r="D103" t="s">
         <v>10</v>
       </c>
-      <c r="E103" s="23">
+      <c r="E103" s="24">
         <v>-8</v>
       </c>
-      <c r="F103" s="23">
+      <c r="F103" s="24">
         <v>2</v>
       </c>
       <c r="G103" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="104" spans="1:7" ht="30">
+      <c r="H103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" ht="30">
       <c r="A104" t="s">
         <v>90</v>
       </c>
@@ -8863,17 +9107,20 @@
       <c r="D104" t="s">
         <v>10</v>
       </c>
-      <c r="E104" s="23">
+      <c r="E104" s="24">
         <v>6</v>
       </c>
-      <c r="F104" s="23">
+      <c r="F104" s="24">
         <v>5</v>
       </c>
       <c r="G104" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="105" spans="1:7" ht="30">
+      <c r="H104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="30">
       <c r="A105" t="s">
         <v>90</v>
       </c>
@@ -8887,17 +9134,20 @@
       <c r="D105" t="s">
         <v>14</v>
       </c>
-      <c r="E105" s="23">
+      <c r="E105" s="24">
         <v>5</v>
       </c>
-      <c r="F105" s="23">
+      <c r="F105" s="24">
         <v>1</v>
       </c>
       <c r="G105" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="106" spans="1:7" ht="30">
+      <c r="H105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" ht="30">
       <c r="A106" t="s">
         <v>90</v>
       </c>
@@ -8911,17 +9161,20 @@
       <c r="D106" t="s">
         <v>14</v>
       </c>
-      <c r="E106" s="23">
+      <c r="E106" s="24">
         <v>5</v>
       </c>
-      <c r="F106" s="23">
+      <c r="F106" s="24">
         <v>2</v>
       </c>
       <c r="G106" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="107" spans="1:7" ht="30">
+      <c r="H106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" ht="30">
       <c r="A107" t="s">
         <v>90</v>
       </c>
@@ -8935,17 +9188,20 @@
       <c r="D107" t="s">
         <v>14</v>
       </c>
-      <c r="E107" s="23">
+      <c r="E107" s="24">
         <v>-2</v>
       </c>
-      <c r="F107" s="23">
+      <c r="F107" s="24">
         <v>-2</v>
       </c>
       <c r="G107" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="108" spans="1:7" ht="30">
+      <c r="H107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="30">
       <c r="A108" t="s">
         <v>90</v>
       </c>
@@ -8959,17 +9215,20 @@
       <c r="D108" t="s">
         <v>14</v>
       </c>
-      <c r="E108" s="23">
+      <c r="E108" s="24">
         <v>-2</v>
       </c>
-      <c r="F108" s="23">
+      <c r="F108" s="24">
         <v>-2</v>
       </c>
       <c r="G108" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="109" spans="1:7" ht="30">
+      <c r="H108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" ht="30">
       <c r="A109" t="s">
         <v>90</v>
       </c>
@@ -8983,17 +9242,20 @@
       <c r="D109" t="s">
         <v>14</v>
       </c>
-      <c r="E109" s="23">
+      <c r="E109" s="24">
         <v>4</v>
       </c>
-      <c r="F109" s="23">
+      <c r="F109" s="24">
         <v>1</v>
       </c>
       <c r="G109" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="110" spans="1:7" ht="30">
+      <c r="H109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" ht="30">
       <c r="A110" t="s">
         <v>90</v>
       </c>
@@ -9007,17 +9269,20 @@
       <c r="D110" t="s">
         <v>14</v>
       </c>
-      <c r="E110" s="23">
+      <c r="E110" s="24">
         <v>9</v>
       </c>
-      <c r="F110" s="23">
+      <c r="F110" s="24">
         <v>3</v>
       </c>
       <c r="G110" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="111" spans="1:7" ht="30">
+      <c r="H110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" ht="30">
       <c r="A111" t="s">
         <v>90</v>
       </c>
@@ -9031,17 +9296,20 @@
       <c r="D111" t="s">
         <v>14</v>
       </c>
-      <c r="E111" s="23">
+      <c r="E111" s="24">
         <v>-9</v>
       </c>
-      <c r="F111" s="23">
+      <c r="F111" s="24">
         <v>-3</v>
       </c>
       <c r="G111" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="112" spans="1:7" ht="30">
+      <c r="H111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" ht="30">
       <c r="A112" t="s">
         <v>91</v>
       </c>
@@ -9055,17 +9323,20 @@
       <c r="D112" t="s">
         <v>10</v>
       </c>
-      <c r="E112" s="23">
+      <c r="E112" s="24">
         <v>9</v>
       </c>
-      <c r="F112" s="23">
+      <c r="F112" s="24">
         <v>7</v>
       </c>
       <c r="G112" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="113" spans="1:7" ht="30">
+      <c r="H112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" ht="30">
       <c r="A113" t="s">
         <v>91</v>
       </c>
@@ -9079,17 +9350,20 @@
       <c r="D113" t="s">
         <v>10</v>
       </c>
-      <c r="E113" s="23">
+      <c r="E113" s="24">
         <v>8</v>
       </c>
-      <c r="F113" s="23">
+      <c r="F113" s="24">
         <v>7</v>
       </c>
       <c r="G113" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="114" spans="1:7" ht="30">
+      <c r="H113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" ht="30">
       <c r="A114" t="s">
         <v>91</v>
       </c>
@@ -9103,17 +9377,20 @@
       <c r="D114" t="s">
         <v>10</v>
       </c>
-      <c r="E114" s="23">
+      <c r="E114" s="24">
         <v>7</v>
       </c>
-      <c r="F114" s="23">
+      <c r="F114" s="24">
         <v>7</v>
       </c>
       <c r="G114" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="115" spans="1:7" ht="30">
+      <c r="H114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" ht="30">
       <c r="A115" t="s">
         <v>91</v>
       </c>
@@ -9127,17 +9404,20 @@
       <c r="D115" t="s">
         <v>10</v>
       </c>
-      <c r="E115" s="23">
+      <c r="E115" s="24">
         <v>6</v>
       </c>
-      <c r="F115" s="23">
+      <c r="F115" s="24">
         <v>7</v>
       </c>
       <c r="G115" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="116" spans="1:7" ht="30">
+      <c r="H115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" ht="30">
       <c r="A116" t="s">
         <v>91</v>
       </c>
@@ -9151,17 +9431,20 @@
       <c r="D116" t="s">
         <v>10</v>
       </c>
-      <c r="E116" s="23">
-        <v>0</v>
-      </c>
-      <c r="F116" s="23">
+      <c r="E116" s="24">
+        <v>0</v>
+      </c>
+      <c r="F116" s="24">
         <v>0</v>
       </c>
       <c r="G116" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="117" spans="1:7" ht="30">
+      <c r="H116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" ht="30">
       <c r="A117" t="s">
         <v>91</v>
       </c>
@@ -9175,17 +9458,20 @@
       <c r="D117" t="s">
         <v>14</v>
       </c>
-      <c r="E117" s="23">
+      <c r="E117" s="24">
         <v>-4</v>
       </c>
-      <c r="F117" s="23">
+      <c r="F117" s="24">
         <v>-2</v>
       </c>
       <c r="G117" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="118" spans="1:7" ht="30">
+      <c r="H117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" ht="30">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -9199,17 +9485,20 @@
       <c r="D118" t="s">
         <v>14</v>
       </c>
-      <c r="E118" s="23">
+      <c r="E118" s="24">
         <v>2</v>
       </c>
-      <c r="F118" s="23">
+      <c r="F118" s="24">
         <v>2</v>
       </c>
       <c r="G118" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="119" spans="1:7" ht="30">
+      <c r="H118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" ht="30">
       <c r="A119" t="s">
         <v>91</v>
       </c>
@@ -9223,17 +9512,20 @@
       <c r="D119" t="s">
         <v>14</v>
       </c>
-      <c r="E119" s="23">
-        <v>0</v>
-      </c>
-      <c r="F119" s="23">
+      <c r="E119" s="24">
+        <v>0</v>
+      </c>
+      <c r="F119" s="24">
         <v>0</v>
       </c>
       <c r="G119" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="120" spans="1:7" ht="30">
+      <c r="H119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" ht="30">
       <c r="A120" t="s">
         <v>91</v>
       </c>
@@ -9247,17 +9539,20 @@
       <c r="D120" t="s">
         <v>14</v>
       </c>
-      <c r="E120" s="23">
+      <c r="E120" s="24">
         <v>-2</v>
       </c>
-      <c r="F120" s="23">
+      <c r="F120" s="24">
         <v>-1</v>
       </c>
       <c r="G120" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="121" spans="1:7" ht="30">
+      <c r="H120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" ht="30">
       <c r="A121" t="s">
         <v>91</v>
       </c>
@@ -9271,17 +9566,20 @@
       <c r="D121" t="s">
         <v>14</v>
       </c>
-      <c r="E121" s="23">
+      <c r="E121" s="24">
         <v>4</v>
       </c>
-      <c r="F121" s="23">
+      <c r="F121" s="24">
         <v>4</v>
       </c>
       <c r="G121" s="14" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="122" spans="1:7" ht="30">
+      <c r="H121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" ht="30">
       <c r="A122" t="s">
         <v>92</v>
       </c>
@@ -9295,17 +9593,20 @@
       <c r="D122" t="s">
         <v>10</v>
       </c>
-      <c r="E122" s="23">
+      <c r="E122" s="24">
         <v>-8</v>
       </c>
-      <c r="F122" s="23">
+      <c r="F122" s="24">
         <v>-4</v>
       </c>
       <c r="G122" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="123" spans="1:7" ht="30">
+      <c r="H122">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" ht="30">
       <c r="A123" t="s">
         <v>92</v>
       </c>
@@ -9319,17 +9620,20 @@
       <c r="D123" t="s">
         <v>10</v>
       </c>
-      <c r="E123" s="23">
+      <c r="E123" s="24">
         <v>-6</v>
       </c>
-      <c r="F123" s="23">
+      <c r="F123" s="24">
         <v>-5</v>
       </c>
       <c r="G123" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="124" spans="1:7" ht="30">
+      <c r="H123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" ht="30">
       <c r="A124" t="s">
         <v>92</v>
       </c>
@@ -9343,17 +9647,20 @@
       <c r="D124" t="s">
         <v>10</v>
       </c>
-      <c r="E124" s="23">
+      <c r="E124" s="24">
         <v>-7</v>
       </c>
-      <c r="F124" s="23">
+      <c r="F124" s="24">
         <v>-4</v>
       </c>
       <c r="G124" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="125" spans="1:7" ht="30">
+      <c r="H124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" ht="30">
       <c r="A125" t="s">
         <v>92</v>
       </c>
@@ -9367,17 +9674,20 @@
       <c r="D125" t="s">
         <v>10</v>
       </c>
-      <c r="E125" s="23">
+      <c r="E125" s="24">
         <v>-6</v>
       </c>
-      <c r="F125" s="23">
+      <c r="F125" s="24">
         <v>-3</v>
       </c>
       <c r="G125" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="126" spans="1:7" ht="30">
+      <c r="H125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" ht="30">
       <c r="A126" t="s">
         <v>92</v>
       </c>
@@ -9391,17 +9701,20 @@
       <c r="D126" t="s">
         <v>10</v>
       </c>
-      <c r="E126" s="23">
+      <c r="E126" s="24">
         <v>-5</v>
       </c>
-      <c r="F126" s="23">
+      <c r="F126" s="24">
         <v>-4</v>
       </c>
       <c r="G126" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="127" spans="1:7" ht="30">
+      <c r="H126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" ht="30">
       <c r="A127" t="s">
         <v>92</v>
       </c>
@@ -9415,17 +9728,20 @@
       <c r="D127" t="s">
         <v>10</v>
       </c>
-      <c r="E127" s="23">
+      <c r="E127" s="24">
         <v>-5</v>
       </c>
-      <c r="F127" s="23">
+      <c r="F127" s="24">
         <v>-4</v>
       </c>
       <c r="G127" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="128" spans="1:7" ht="30">
+      <c r="H127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" ht="30">
       <c r="A128" t="s">
         <v>92</v>
       </c>
@@ -9439,17 +9755,20 @@
       <c r="D128" t="s">
         <v>14</v>
       </c>
-      <c r="E128" s="23">
+      <c r="E128" s="24">
         <v>6</v>
       </c>
-      <c r="F128" s="23">
+      <c r="F128" s="24">
         <v>2</v>
       </c>
       <c r="G128" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="129" spans="1:7" ht="30">
+      <c r="H128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" ht="30">
       <c r="A129" t="s">
         <v>92</v>
       </c>
@@ -9463,17 +9782,20 @@
       <c r="D129" t="s">
         <v>14</v>
       </c>
-      <c r="E129" s="23">
+      <c r="E129" s="24">
         <v>-8</v>
       </c>
-      <c r="F129" s="23">
+      <c r="F129" s="24">
         <v>-2</v>
       </c>
       <c r="G129" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="130" spans="1:7" ht="30">
+      <c r="H129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" ht="30">
       <c r="A130" t="s">
         <v>92</v>
       </c>
@@ -9487,17 +9809,20 @@
       <c r="D130" t="s">
         <v>14</v>
       </c>
-      <c r="E130" s="23">
+      <c r="E130" s="24">
         <v>5</v>
       </c>
-      <c r="F130" s="23">
+      <c r="F130" s="24">
         <v>1</v>
       </c>
       <c r="G130" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="131" spans="1:7" ht="30">
+      <c r="H130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" ht="30">
       <c r="A131" t="s">
         <v>92</v>
       </c>
@@ -9511,17 +9836,20 @@
       <c r="D131" t="s">
         <v>14</v>
       </c>
-      <c r="E131" s="23">
+      <c r="E131" s="24">
         <v>4</v>
       </c>
-      <c r="F131" s="23">
+      <c r="F131" s="24">
         <v>1</v>
       </c>
       <c r="G131" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="132" spans="1:7" ht="30">
+      <c r="H131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" ht="30">
       <c r="A132" t="s">
         <v>92</v>
       </c>
@@ -9535,17 +9863,20 @@
       <c r="D132" t="s">
         <v>14</v>
       </c>
-      <c r="E132" s="23">
+      <c r="E132" s="24">
         <v>-7</v>
       </c>
-      <c r="F132" s="23">
+      <c r="F132" s="24">
         <v>-3</v>
       </c>
       <c r="G132" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="133" spans="1:7" ht="30">
+      <c r="H132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" ht="30">
       <c r="A133" t="s">
         <v>92</v>
       </c>
@@ -9559,17 +9890,20 @@
       <c r="D133" t="s">
         <v>14</v>
       </c>
-      <c r="E133" s="23">
+      <c r="E133" s="24">
         <v>-7</v>
       </c>
-      <c r="F133" s="23">
+      <c r="F133" s="24">
         <v>-3</v>
       </c>
       <c r="G133" s="14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="134" spans="1:7" ht="30">
+      <c r="H133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" ht="30">
       <c r="A134" t="s">
         <v>93</v>
       </c>
@@ -9583,17 +9917,20 @@
       <c r="D134" t="s">
         <v>10</v>
       </c>
-      <c r="E134" s="23">
+      <c r="E134" s="24">
         <v>-5</v>
       </c>
-      <c r="F134" s="23">
+      <c r="F134" s="24">
         <v>-2</v>
       </c>
       <c r="G134" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="135" spans="1:7" ht="30">
+      <c r="H134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" ht="30">
       <c r="A135" t="s">
         <v>93</v>
       </c>
@@ -9607,17 +9944,20 @@
       <c r="D135" t="s">
         <v>10</v>
       </c>
-      <c r="E135" s="23">
+      <c r="E135" s="24">
         <v>-4</v>
       </c>
-      <c r="F135" s="23">
+      <c r="F135" s="24">
         <v>-2</v>
       </c>
       <c r="G135" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="136" spans="1:7" ht="30">
+      <c r="H135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" ht="30">
       <c r="A136" t="s">
         <v>93</v>
       </c>
@@ -9631,17 +9971,20 @@
       <c r="D136" t="s">
         <v>10</v>
       </c>
-      <c r="E136" s="23">
-        <v>0</v>
-      </c>
-      <c r="F136" s="23">
+      <c r="E136" s="24">
+        <v>0</v>
+      </c>
+      <c r="F136" s="24">
         <v>0</v>
       </c>
       <c r="G136" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="137" spans="1:7" ht="30">
+      <c r="H136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" ht="30">
       <c r="A137" t="s">
         <v>93</v>
       </c>
@@ -9655,17 +9998,20 @@
       <c r="D137" t="s">
         <v>10</v>
       </c>
-      <c r="E137" s="23">
-        <v>0</v>
-      </c>
-      <c r="F137" s="23">
+      <c r="E137" s="24">
+        <v>0</v>
+      </c>
+      <c r="F137" s="24">
         <v>0</v>
       </c>
       <c r="G137" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="138" spans="1:7" ht="30">
+      <c r="H137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" ht="30">
       <c r="A138" t="s">
         <v>93</v>
       </c>
@@ -9679,17 +10025,20 @@
       <c r="D138" t="s">
         <v>10</v>
       </c>
-      <c r="E138" s="23">
-        <v>0</v>
-      </c>
-      <c r="F138" s="23">
+      <c r="E138" s="24">
+        <v>0</v>
+      </c>
+      <c r="F138" s="24">
         <v>0</v>
       </c>
       <c r="G138" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="139" spans="1:7" ht="30">
+      <c r="H138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" ht="30">
       <c r="A139" t="s">
         <v>93</v>
       </c>
@@ -9703,17 +10052,20 @@
       <c r="D139" t="s">
         <v>10</v>
       </c>
-      <c r="E139" s="23">
-        <v>0</v>
-      </c>
-      <c r="F139" s="23">
+      <c r="E139" s="24">
+        <v>0</v>
+      </c>
+      <c r="F139" s="24">
         <v>0</v>
       </c>
       <c r="G139" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="140" spans="1:7" ht="30">
+      <c r="H139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" ht="30">
       <c r="A140" t="s">
         <v>93</v>
       </c>
@@ -9727,17 +10079,20 @@
       <c r="D140" t="s">
         <v>14</v>
       </c>
-      <c r="E140" s="23">
+      <c r="E140" s="24">
         <v>7</v>
       </c>
-      <c r="F140" s="23">
+      <c r="F140" s="24">
         <v>4</v>
       </c>
       <c r="G140" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="141" spans="1:7" ht="30">
+      <c r="H140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" ht="30">
       <c r="A141" t="s">
         <v>93</v>
       </c>
@@ -9751,17 +10106,20 @@
       <c r="D141" t="s">
         <v>14</v>
       </c>
-      <c r="E141" s="23">
+      <c r="E141" s="24">
         <v>6</v>
       </c>
-      <c r="F141" s="23">
+      <c r="F141" s="24">
         <v>4</v>
       </c>
       <c r="G141" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="142" spans="1:7" ht="30">
+      <c r="H141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" ht="30">
       <c r="A142" t="s">
         <v>93</v>
       </c>
@@ -9775,17 +10133,20 @@
       <c r="D142" t="s">
         <v>14</v>
       </c>
-      <c r="E142" s="23">
+      <c r="E142" s="24">
         <v>-2</v>
       </c>
-      <c r="F142" s="23">
+      <c r="F142" s="24">
         <v>2</v>
       </c>
       <c r="G142" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="143" spans="1:7" ht="30">
+      <c r="H142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" ht="30">
       <c r="A143" t="s">
         <v>93</v>
       </c>
@@ -9799,17 +10160,20 @@
       <c r="D143" t="s">
         <v>14</v>
       </c>
-      <c r="E143" s="23">
+      <c r="E143" s="24">
         <v>-3</v>
       </c>
-      <c r="F143" s="23">
+      <c r="F143" s="24">
         <v>3</v>
       </c>
       <c r="G143" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="144" spans="1:7" ht="30">
+      <c r="H143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" ht="30">
       <c r="A144" t="s">
         <v>93</v>
       </c>
@@ -9823,17 +10187,20 @@
       <c r="D144" t="s">
         <v>14</v>
       </c>
-      <c r="E144" s="23">
+      <c r="E144" s="24">
         <v>5</v>
       </c>
-      <c r="F144" s="23">
+      <c r="F144" s="24">
         <v>5</v>
       </c>
       <c r="G144" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="145" spans="1:7" ht="30">
+      <c r="H144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" ht="30">
       <c r="A145" t="s">
         <v>93</v>
       </c>
@@ -9847,17 +10214,20 @@
       <c r="D145" t="s">
         <v>14</v>
       </c>
-      <c r="E145" s="23">
+      <c r="E145" s="24">
         <v>-6</v>
       </c>
-      <c r="F145" s="23">
+      <c r="F145" s="24">
         <v>-2</v>
       </c>
       <c r="G145" s="14" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="146" spans="1:7" ht="30">
+      <c r="H145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" ht="30">
       <c r="A146" t="s">
         <v>94</v>
       </c>
@@ -9871,112 +10241,143 @@
       <c r="D146" t="s">
         <v>14</v>
       </c>
-      <c r="E146" s="23">
-        <v>10</v>
-      </c>
-      <c r="F146" s="23">
+      <c r="E146" s="24">
+        <v>10</v>
+      </c>
+      <c r="F146" s="24">
         <v>8</v>
       </c>
       <c r="G146" s="14" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="147" spans="1:7">
+      <c r="H146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8">
       <c r="B147" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C147, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E147" s="24"/>
+      <c r="F147" s="24"/>
       <c r="G147" s="14"/>
     </row>
-    <row r="148" spans="1:7">
+    <row r="148" spans="1:8">
       <c r="B148" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C148, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E148" s="24"/>
+      <c r="F148" s="24"/>
       <c r="G148" s="14"/>
     </row>
-    <row r="149" spans="1:7">
+    <row r="149" spans="1:8">
       <c r="B149" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C149, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E149" s="24"/>
+      <c r="F149" s="24"/>
       <c r="G149" s="14"/>
     </row>
-    <row r="150" spans="1:7">
+    <row r="150" spans="1:8">
       <c r="B150" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C150, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E150" s="24"/>
+      <c r="F150" s="24"/>
       <c r="G150" s="14"/>
     </row>
-    <row r="151" spans="1:7">
+    <row r="151" spans="1:8">
       <c r="B151" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C151, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E151" s="24"/>
+      <c r="F151" s="24"/>
       <c r="G151" s="14"/>
     </row>
-    <row r="152" spans="1:7">
+    <row r="152" spans="1:8">
       <c r="B152" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C152, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E152" s="24"/>
+      <c r="F152" s="24"/>
       <c r="G152" s="14"/>
     </row>
-    <row r="153" spans="1:7">
+    <row r="153" spans="1:8">
       <c r="B153" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C153, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E153" s="24"/>
+      <c r="F153" s="24"/>
       <c r="G153" s="14"/>
     </row>
-    <row r="154" spans="1:7">
+    <row r="154" spans="1:8">
       <c r="B154" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C154, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E154" s="24"/>
+      <c r="F154" s="24"/>
       <c r="G154" s="14"/>
     </row>
-    <row r="155" spans="1:7">
+    <row r="155" spans="1:8">
       <c r="B155" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C155, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E155" s="24"/>
+      <c r="F155" s="24"/>
       <c r="G155" s="14"/>
     </row>
-    <row r="156" spans="1:7">
+    <row r="156" spans="1:8">
       <c r="B156" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C156, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E156" s="24"/>
+      <c r="F156" s="24"/>
       <c r="G156" s="14"/>
     </row>
-    <row r="157" spans="1:7">
+    <row r="157" spans="1:8">
       <c r="B157" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C157, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E157" s="24"/>
+      <c r="F157" s="24"/>
       <c r="G157" s="14"/>
     </row>
-    <row r="158" spans="1:7">
+    <row r="158" spans="1:8">
       <c r="B158" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C158, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E158" s="24"/>
+      <c r="F158" s="24"/>
       <c r="G158" s="14"/>
     </row>
-    <row r="159" spans="1:7">
+    <row r="159" spans="1:8">
       <c r="B159" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C159, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E159" s="24"/>
+      <c r="F159" s="24"/>
       <c r="G159" s="14"/>
     </row>
-    <row r="160" spans="1:7">
+    <row r="160" spans="1:8">
       <c r="B160" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C160, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E160" s="24"/>
+      <c r="F160" s="24"/>
       <c r="G160" s="14"/>
     </row>
     <row r="161" spans="2:7">
@@ -9984,6 +10385,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C161, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E161" s="24"/>
+      <c r="F161" s="24"/>
       <c r="G161" s="14"/>
     </row>
     <row r="162" spans="2:7">
@@ -9991,6 +10394,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C162, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E162" s="24"/>
+      <c r="F162" s="24"/>
       <c r="G162" s="14"/>
     </row>
     <row r="163" spans="2:7">
@@ -9998,6 +10403,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C163, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E163" s="24"/>
+      <c r="F163" s="24"/>
       <c r="G163" s="14"/>
     </row>
     <row r="164" spans="2:7">
@@ -10005,6 +10412,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C164, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E164" s="24"/>
+      <c r="F164" s="24"/>
       <c r="G164" s="14"/>
     </row>
     <row r="165" spans="2:7">
@@ -10012,6 +10421,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C165, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E165" s="24"/>
+      <c r="F165" s="24"/>
       <c r="G165" s="14"/>
     </row>
     <row r="166" spans="2:7">
@@ -10019,6 +10430,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C166, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E166" s="24"/>
+      <c r="F166" s="24"/>
       <c r="G166" s="14"/>
     </row>
     <row r="167" spans="2:7">
@@ -10026,6 +10439,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C167, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E167" s="24"/>
+      <c r="F167" s="24"/>
       <c r="G167" s="14"/>
     </row>
     <row r="168" spans="2:7">
@@ -10033,6 +10448,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C168, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E168" s="24"/>
+      <c r="F168" s="24"/>
       <c r="G168" s="14"/>
     </row>
     <row r="169" spans="2:7">
@@ -10040,6 +10457,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C169, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E169" s="24"/>
+      <c r="F169" s="24"/>
       <c r="G169" s="14"/>
     </row>
     <row r="170" spans="2:7">
@@ -10047,6 +10466,8 @@
         <f>IFERROR(_xlfn.XLOOKUP(C170, tblActors[nome], tblActors[actor_id], ""), "")</f>
         <v/>
       </c>
+      <c r="E170" s="24"/>
+      <c r="F170" s="24"/>
       <c r="G170" s="14"/>
     </row>
     <row r="171" spans="2:7">

</xml_diff>